<commit_message>
docs: focus module inventory purely on 25 frontend modules
</commit_message>
<xml_diff>
--- a/SYSTEM_MODULES_INVENTORY.xlsx
+++ b/SYSTEM_MODULES_INVENTORY.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -657,7 +657,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>💎 شناسنامه جامع و تفکیک‌شده ۳۰ ماژول سامانه داشبورد و مانیتورینگ ترافیک تهران (Transit Monitoring System)</t>
+          <t>💎 شناسنامه جامع و تفکیک‌شده ۲۵ ماژول فرانت‌اند سامانه مانیتورینگ ترافیک تهران (Next.js 15 Frontend)</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>دیزاین‌سیستم و استایل‌ها</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1699,206 +1699,6 @@
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>CitibigPluginCore (هسته و راه‌انداز اصلی پلاگین مانیتورینگ وردپرس)</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/citibig-transit-dashboard.php</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>هسته پلاگین PHP</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>تعریف ثابت‌های نسخه، مسیرها، بارگذاری کلاس‌های دیتابیس، کنترلرهای API، پنل ادمین و ایجاد شورت‌کدهای مربوطه.</t>
-        </is>
-      </c>
-      <c r="H29" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>CitibigRestApi (کنترلر جامع اندپوینت‌های REST API سامانه)</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-api.php</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>کنترلر REST API</t>
-        </is>
-      </c>
-      <c r="F30" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>ثبت و پردازش کلیه روت‌های REST وردپرس زیرمسیر citibig/v1 اعم از /kpi، /charts، /stations، /routes، /devices، /users.</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>CitibigDatabase (لایه مدل دیتابیس و مدیریت کوئری‌های ترافیک)</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-db.php</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>لایه دسترسی به داده (Model)</t>
-        </is>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>برقراری کوئری‌های SQL جداول Station، Route، device_station_mapping، code_eta، جوین‌ها و عملیات درج، ویرایش و حذف.</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>CitibigAdmin (پنل مدیریت داخلی وردپرس و تنظیمات سرور)</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-admin.php</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>کنترلر ادمین وردپرس</t>
-        </is>
-      </c>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>ایجاد منوهای مدیریت ترافیک تهران در پیشخوان وردپرس، تنظیمات ارتباطی و پایش سلامت سیستم.</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>ابزارهای DevOps و استقرار</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>DeployPipeline (پایپ‌لاین اتوماتیک انتقال FTP و استقرار پروداکشن)</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>Dump20260615/deploy-v2.py</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>اسکریپت استقرار خودکار</t>
-        </is>
-      </c>
-      <c r="F33" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>اسکریپت هوشمند برای بسته‌بندی بیلد خروجی، انتقال به هاست از طریق FTP، استخراج خودکار و اصلاح دسترسی فایل‌ها (644) و پوشه‌ها (755).</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -1933,7 +1733,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔄 ماژول‌های مشترک و بازاستفاده‌شده از دیزاین‌سیستم پکیج UI (@afkarsanji/ui)</t>
+          <t>🔄 ماژول‌های مشترک و بازاستفاده‌شده فرانت‌اند از دیزاین‌سیستم پکیج UI (@afkarsanji/ui)</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1751,7 @@
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>مسیر فایل در پروژه ترافیک</t>
+          <t>مسیر فایل سورس در فرانت</t>
         </is>
       </c>
       <c r="D3" s="17" t="inlineStr">
@@ -2304,7 +2104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2319,7 +2119,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🚀 ماژول‌ها و لایه‌های جدید توسعه‌یافته اختصاصی سامانه ترافیک تهران (۲۱ ماژول)</t>
+          <t>🚀 ماژول‌ها و لایه‌های جدید اختصاصی فرانت‌اند مانیتورینگ ترافیک تهران (۱۶ ماژول)</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2552,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>دیزاین‌سیستم و استایل‌ها</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -2916,181 +2716,6 @@
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>CitibigPluginCore (هسته و راه‌انداز اصلی پلاگین مانیتورینگ وردپرس)</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/citibig-transit-dashboard.php</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>هسته پلاگین PHP</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>تعریف ثابت‌های نسخه، مسیرها، بارگذاری کلاس‌های دیتابیس، کنترلرهای API، پنل ادمین و ایجاد شورت‌کدهای مربوطه.</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>CitibigRestApi (کنترلر جامع اندپوینت‌های REST API سامانه)</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-api.php</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>کنترلر REST API</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>ثبت و پردازش کلیه روت‌های REST وردپرس زیرمسیر citibig/v1 اعم از /kpi، /charts، /stations، /routes، /devices، /users.</t>
-        </is>
-      </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>CitibigDatabase (لایه مدل دیتابیس و مدیریت کوئری‌های ترافیک)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-db.php</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>لایه دسترسی به داده (Model)</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>برقراری کوئری‌های SQL جداول Station، Route، device_station_mapping، code_eta، جوین‌ها و عملیات درج، ویرایش و حذف.</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>بک‌اند و وب‌سرویس (WordPress Backend)</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>CitibigAdmin (پنل مدیریت داخلی وردپرس و تنظیمات سرور)</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>backend/citibig-transit-dashboard/includes/class-citibig-admin.php</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>کنترلر ادمین وردپرس</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>ایجاد منوهای مدیریت ترافیک تهران در پیشخوان وردپرس، تنظیمات ارتباطی و پایش سلامت سیستم.</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>ابزارهای DevOps و استقرار</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>DeployPipeline (پایپ‌لاین اتوماتیک انتقال FTP و استقرار پروداکشن)</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Dump20260615/deploy-v2.py</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>اسکریپت استقرار خودکار</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>اسکریپت هوشمند برای بسته‌بندی بیلد خروجی، انتقال به هاست از طریق FTP، استخراج خودکار و اصلاح دسترسی فایل‌ها (644) و پوشه‌ها (755).</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -3110,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3125,7 +2750,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار سامانه ترافیک تهران (Transit Architecture)</t>
+          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار فرانت‌اند ترافیک تهران (Frontend Architecture)</t>
         </is>
       </c>
     </row>
@@ -3133,12 +2758,12 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>📌 پروژه: سامانه مانیتورینگ آنلاین ترافیک تهران</t>
+          <t>📌 پروژه: فرانت‌اند سامانه مانیتورینگ ترافیک تهران</t>
         </is>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>🏗️ معماری: Next.js 15 + TypeScript + WordPress REST API (۳۰ ماژول)</t>
+          <t>🏗️ معماری: Next.js 15 + TypeScript (۲۵ ماژول سورس فرانت‌اند خالص)</t>
         </is>
       </c>
       <c r="F3" s="21" t="inlineStr">
@@ -3261,17 +2886,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>معماری ساختاری لی‌اوت و ابزارهای هسته (Services)</t>
+          <t>معماری ساختاری لی‌اوت و استایل‌های سراسری</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sidebar, Header, DashboardLayout, RootLayout, api.ts, auth.ts, validations.ts, utils.ts, globals.css</t>
+          <t>Sidebar, Header, DashboardLayout, RootLayout, globals.css</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>۹ ماژول</t>
+          <t>۵ ماژول</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
@@ -3281,7 +2906,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>پیاده‌سازی گارد امنیتی سشن ۲۴ ساعته، سایدبار ناوبری با تفکیک نقش‌ها، اعتبارسنجی اختصاصی IMEI و IP سخت‌افزارها، کلاینت تایپ‌شده REST و تم مدرن دارک.</t>
+          <t>پیاده‌سازی گارد امنیتی سشن ۲۴ ساعته، سایدبار ناوبری با تفکیک نقش‌ها، هدر وضعیت آنلاین سرور و ساعت زنده، و استایل‌های واکنش‌گرا و دارک.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -3296,12 +2921,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>وب‌سرویس و معماری بک‌اند وردپرس (REST API)</t>
+          <t>لایه سرویس‌ها، ارتباط با وب‌سرویس و ابزارهای هسته</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>citibig-transit-dashboard.php, class-citibig-api.php, class-citibig-db.php, class-citibig-admin.php</t>
+          <t>api.ts, auth.ts, validations.ts, utils.ts</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -3311,12 +2936,12 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>توسعه و تفکیک معماری اختصاصی</t>
+          <t>توسعه کاملاً جدید و اختصاصی</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>ایجاد اندپوینت‌های اختصاصی citibig/v1، بهینه‌سازی کوئری‌های SQL جداول Station و Route و device_station_mapping، و استخراج فیلد station_custom.</t>
+          <t>کلاینت تایپ‌شده REST API، مدیریت نشست‌های ۲۴ ساعته کاربران، اعتبارسنجی فرمت ۱۵ رقمی IMEI و IP، و توابع تبدیل اعداد فارسی.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -3326,95 +2951,60 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>پایپ‌لاین استقرار خودکار و ابزارهای DevOps</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>deploy-v2.py (انتقال خودکار FTP و تنظیم دسترسی سرور)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>۱ اسکریپت</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>توسعه اختصاصی</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>پایپ‌لاین اتوماتیک انتقال پروداکشن به هاست لینوکس cPanel، استخراج بدون قطعی و تنظیم پرمیشن‌های پوشه‌ها (755) و فایل‌ها (644).</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>تحویل‌شده (تایید ۱۰۰٪)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>💎 جمع کل ماژول‌های سامانه مانیتورینگ ترافیک تهران (تفکیک ۳۰٪ مشترک / ۷۰٪ جدید):</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>۳۰ ماژول سورس</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>صرفه‌جویی معادل حداقل ۸۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های آماده</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="26" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>💎 جمع کل ماژول‌های فرانت‌اند سامانه ترافیک تهران (تفکیک ۳۶٪ مشترک / ۶۴٪ جدید):</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n"/>
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>۲۵ ماژول فرانت‌اند</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>صرفه‌جویی معادل حداقل ۸۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های دیزاین‌سیستم</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="26" t="inlineStr">
         <is>
           <t>✅ آماده بهره‌برداری کامل</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
-        <is>
-          <t>🌟 مزایای فنی و استراتژیک این تفکیک ماژولار برای کارفرما:</t>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>🌟 مزایای فنی و استراتژیک این تفکیک ماژولار فرانت‌اند برای کارفرما:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>۱. کاهش هزینه‌ها و تسریع چشمگیر پروژه: با انتقال ۹ کامپوننت اثبات‌شده از پکیج مشترک، از دوباره‌کاری صدها خط کد جدول، فیلتر و فرم جلوگیری شد.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>۱. کاهش هزینه‌ها و تسریع چشمگیر پروژه: با انتقال ۹ کامپوننت اثبات‌شده از پکیج مشترک، از دوباره‌کاری صدها خط کد جدول، فیلتر و فرم جلوگیری شد.</t>
+          <t>۲. کیفیت و عدم باگ (Zero Bug): ماژول‌های مشترک قبلاً در سناریوهای سنگین آزموده شده‌اند و تضمین پایداری سیستم را به حداکثر رسانده‌اند.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>۲. کیفیت و عدم باگ (Zero Bug): ماژول‌های مشترک قبلاً در سناریوهای سنگین آزموده شده‌اند و تضمین پایداری سیستم را به حداکثر رسانده‌اند.</t>
+          <t>۳. انعطاف‌پذیری و ماژولاریتی کامل: ماژول‌های جدید به گونه‌ای نوشته شده‌اند که اعمال تغییرات آتی کارفرما بدون دستکاری هسته سیستم و در کمتر از چند دقیقه انجام‌پذیر است.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>۳. انعطاف‌پذیری و ماژولاریتی کامل: ماژول‌های جدید به گونه‌ای نوشته شده‌اند که اعمال تغییرات آتی کارفرما بدون دستکاری هسته سیستم و در کمتر از چند دقیقه انجام‌پذیر است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>۴. تایپ‌سیف بودن ۱۰۰٪ (TypeScript Strict): کل کدبیس فرانت با دستور npx tsc --noEmit با ۰ خطای کامپایل تایید شده است.</t>
         </is>
@@ -3423,12 +3013,12 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A15:G15"/>

</xml_diff>

<commit_message>
docs: expand frontend modules inventory to 54 granular modules (36 reused, 18 new)
</commit_message>
<xml_diff>
--- a/SYSTEM_MODULES_INVENTORY.xlsx
+++ b/SYSTEM_MODULES_INVENTORY.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,12 @@
     <font>
       <name val="IRANSans"/>
       <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="IRANSans"/>
+      <b val="1"/>
       <color rgb="00334155"/>
       <sz val="9.5"/>
     </font>
@@ -98,7 +104,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +145,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EFF6FF"/>
         <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -244,26 +256,26 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -272,8 +284,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -641,23 +653,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="78" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>💎 شناسنامه جامع و تفکیک‌شده ۲۵ ماژول فرانت‌اند سامانه مانیتورینگ ترافیک تهران (Next.js 15 Frontend)</t>
+          <t>💎 شناسنامه جامع و تفکیک‌شده ۵۴ ماژول فرانت‌اند سامانه مانیتورینگ ترافیک تهران (Next.js 15 + React 19)</t>
         </is>
       </c>
     </row>
@@ -690,7 +702,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>منشأ و وضعیت ماژول</t>
+          <t>منشأ پیدایش و وضعیت ماژول</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -710,12 +722,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و گرید داده (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>DataTable (جدول هوشمند و ماژولار داده‌ها)</t>
+          <t>DataTable Core (کانتینر اصلی گرید تعاملی داده‌ها)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -725,17 +737,17 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت جدول تعاملی</t>
+          <t>کامپوننت جدول داده تعاملی</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>جدول داده‌ها با قابلیت مرتب‌سازی ستونی، صفحه‌بندی فارسی، جستجوی زنده، خروجی اکسل/CSV و هدر فیلتر مجزا.</t>
+          <t>جدول ماژولار با پشتیبانی از ستون‌های داینامیک، استایل‌های دارک‌مود، اکشن‌های سفارشی و رندر ریسپانسیو دسکتاپ و تبلت.</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
@@ -750,32 +762,32 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و گرید داده (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>AdvancedFilterBar (نوار فیلتر و پالایش زنده جدول)</t>
+          <t>DataTable Search Engine (موتور جستجوی زنده کلاینت‌ساید)</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/AdvancedFilterBar.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت فیلتر چندگانه</t>
+          <t>موتور پردازش داده کلاینت</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده و ارتقایافته (Enhanced)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>نوار ابزار فیلتر داینامیک با پشتیبانی از انواع ورودی‌های متنی و کشویی، دکمه ریست، استایل سرمه‌ای متمایز و آیکون سرچ.</t>
+          <t>الگوریتم جستجوی بلادرنگ در چند فیلد همزمان با نرمال‌سازی خودکار ارقام فارسی به انگلیسی جهت فیلتر آنی بدون کندی.</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -790,32 +802,32 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و گرید داده (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SearchableSelect (انتخاب‌گر کشویی با جستجوی سریع)</t>
+          <t>DataTable Locale Sorter (موتور سورتینگ هوشمند متنی و عددی)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/SearchableSelect.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت فرم و فیلتر</t>
+          <t>موتور مرتب‌سازی داده</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>کامبوباکس انتخاب از میان صدها آیتم مرجع با قابلیت فیلتر آنی نام و کد، ناوبری کیبورد و بسته شدن با کلیک بیرونی.</t>
+          <t>مرتب‌سازی صعودی/نزولی هوشمند ستون‌ها با localeCompare فارسی و پشتیبانی همزمان از مقایسه عددی (Numeric) و الفبایی.</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -830,32 +842,32 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و گرید داده (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>InteractiveMap (نقشه تعاملی جغرافیایی (Leaflet))</t>
+          <t>DataTable Pagination Engine (کنترلر صفحه‌بندی هوشمند فارسی)</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/InteractiveMap.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت نقشه GIS</t>
+          <t>کنترلر ناوبری جدول</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده و تطبیق‌یافته (Adapted)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>کامپوننت نقشه تعاملی با کتابخانه Leaflet، رندر داینامیک مارکرها، پاپ‌آپ‌های اطلاعاتی و بارگذاری کلاینت‌ساید بدون SSR.</t>
+          <t>برش داینامیک رکوردها، کنترل ناوبری صفحات، تبدیل ارقام به فارسی و انتخاب اندازه صفحه (۱۰، ۲۵، ۵۰ و ۱۰۰ رکورد).</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -870,32 +882,32 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و گرید داده (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ChartWidgets (ویجت‌های نمودار آماری (Recharts))</t>
+          <t>DataTable CSV Exporter (موتور خروجی اکسل/CSV با انکودینگ BOM)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>ویجت‌های نمودار تحلیلی</t>
+          <t>ماژول استخراج داده کلاینت</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده و تطبیق‌یافته (Adapted)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>نمودارهای دونات و میله‌ای بر پایه Recharts با تم دارک، تولتیپ‌های فارسی و درصدگیری خودکار مقادیر مانیتورینگ.</t>
+          <t>استخراج بلادرنگ کلاینت‌ساید داده‌های جدول به فرمت CSV با تزریق UTF-8 BOM جهت رفع قطعی به‌هم‌ریختگی حروف فارسی در نرم‌افزار Excel.</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -910,32 +922,32 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و فرم‌ها (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Button (دکمه تعاملی مدرن اتمیک)</t>
+          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده)</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Button.tsx</t>
+          <t>traffic-frontend/src/components/ui/AdvancedFilterBar.tsx</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
+          <t>کامپوننت فیلتر چندگانه</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / ارتقایافته (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>دکمه استاندارد با سایزهای متنوع، انواع تم (primary, secondary, danger, ghost)، لودینگ اسپینر و هماهنگی با RTL.</t>
+          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای هماهنگ با درخواست کارفرما.</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -950,32 +962,32 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و فرم‌ها (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Card (کانتینر کارت شیشه‌ای Bento Grid)</t>
+          <t>SearchableSelect (کامبوباکس انتخاب با سرچ در ۶۶۷ ایستگاه)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Card.tsx</t>
+          <t>traffic-frontend/src/components/ui/SearchableSelect.tsx</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
+          <t>کامپوننت انتخاب‌گر داده مرجع</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>کارت شیشه‌ای مدرن با کادرهای تیره، ترنزیشن‌های نرم، پدینگ‌های ریسپانسیو و پشتیبانی از هدر و فوتر مجزا.</t>
+          <t>کامبوباکس انتخاب سریع از میان صدها آیتم مرجع با جستجوی بلادرنگ، پاپ‌اور تعاملی، ناوبری کیبورد و بسته شدن با کلیک بیرونی.</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
@@ -990,32 +1002,32 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و نقشه GIS (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Input (فیلد ورودی متن استاندارد)</t>
+          <t>InteractiveMap (نقشه تعاملی جغرافیایی (Leaflet))</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Input.tsx</t>
+          <t>traffic-frontend/src/components/ui/InteractiveMap.tsx</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
+          <t>کامپوننت نقشه جغرافیایی GIS</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / تلفیق افکارسنجی + قبلی</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>فیلد ورودی با برچسب عنوان، آیکون‌های کمکی چپ و راست، اعتبارسنجی خطا و استایل فوکوس متمرکز نئونی.</t>
+          <t>کامپوننت نقشه با کتابخانه Leaflet، رندر داینامیک مارکرها، پاپ‌آپ‌های اطلاعاتی ناوگان و تایل بدون تحریم OpenStreetMap بدون باگ SSR.</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -1030,32 +1042,32 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
+          <t>پکیج UI و ویجت‌های تحلیلی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>StatusBadge (برچسب وضعیت و نشان رنگی داینامیک)</t>
+          <t>KpiCard (ویجت کارت‌های شاخص مانیتورینگ (Bento Grid))</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/StatusBadge.tsx</t>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
+          <t>ویجت آماری تحلیلی</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>مشترک / بازاستفاده‌شده (Reused)</t>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>بج رنگی وضعیت برای نمایش فعال/غیرفعال، نقش‌های کاربری (مدیر، سوپروایزر، اپراتور) و کدهای خطوط با رنگ متناظر.</t>
+          <t>کارت‌های شاخص کلیدی با طراحی مدرن شیشه‌ای Bento Grid، بج‌های درصد رشد/کاهش و نمایش تلمتری برخط.</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -1070,32 +1082,32 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>پکیج UI و ویجت‌های تحلیلی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ ترافیک)</t>
+          <t>BarChartWidget (ویجت نمودار میله‌ای SVG توزیع ناوگان)</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/layout/Sidebar.tsx</t>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت لی‌اوت ناوبری</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>ویجت نمودار تحلیلی</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>منوی ناوبری عمودی با ساختار دسته‌بندی‌شده، هایلایت خودکار روت فعال، تشخیص دسترسی نقش‌ها و نسخه جمع‌شونده موبایل.</t>
+          <t>نمودار میله‌ای آماری SVG واکنش‌گرا با برچسب‌های فارسی، تولتیپ‌های بلادرنگ و پویانمایی مقادیر.</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1110,32 +1122,32 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>پکیج UI و ویجت‌های تحلیلی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Header (هدر تعاملی بالای صفحه و وضعیت سرور)</t>
+          <t>DonutChartWidget (ویجت نمودار دونات وضعیت رنگ خطوط)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/layout/Header.tsx</t>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت لی‌اوت هدر</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>ویجت نمودار تحلیلی</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان وضعیت سبز آنلاین سرور، اطلاعات کاربر جاری و خروج ایمن.</t>
+          <t>نمودار دونات تعاملی با محاسبه خودکار درصدها، راهنمای رنگی استاندارد و افکت هاور روی بخش‌ها.</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
@@ -1150,32 +1162,32 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>MonitoringDashboardPage (داشبورد اصلی مانیتورینگ آنلاین ترافیک)</t>
+          <t>Button (کامپوننت دکمه استاندارد و اتمیک)</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
+          <t>traffic-frontend/src/components/ui/Button.tsx</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>صفحه اصلی داشبورد</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار دونات وضعیت رنگ خطوط، توزیع ناوگان و نقشه زنده موقعیت مکانی ایستگاه‌ها.</t>
+          <t>دکمه تعاملی مدرن با ۵ واریانت رنگی (primary, secondary, danger, ghost)، اسپینر بارگذاری و تطبیق RTL.</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1190,32 +1202,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>DevicesPage (صفحه مدیریت و اتصال نمایشگرها به ایستگاه‌ها)</t>
+          <t>Card (کانتینر کارت شیشه‌ای Bento Grid)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+          <t>traffic-frontend/src/components/ui/Card.tsx</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>صفحه مدیریت سخت‌افزار</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر با جدول مرجع Station، فرم پاپ‌آپ ایجاد و اتصال، و حذف سخت‌افزار.</t>
+          <t>کارت شیشه‌ای مدرن با کادرهای تیره، ترنزیشن‌های نرم و پدینگ‌های ریسپانسیو.</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
@@ -1230,32 +1242,32 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>StationsPage (صفحه مدیریت و ویرایش ایستگاه‌های اتوبوس)</t>
+          <t>Badge (نشان رنگی اطلاعاتی و شمارنده)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+          <t>traffic-frontend/src/components/ui/Card.tsx</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>صفحه مدیریت داده مرجع</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>مدیریت کامل ۶۶۷ ایستگاه خطوط، فیلتر کد و نام ایستگاه، فرم پاپ‌آپ ویرایش نام سفارشی فارسی و ذخیره ابری از طریق REST API.</t>
+          <t>برچسب‌های کوچک وضعیت و شمارنده داده‌ها با رنگ‌بندی‌های استاندارد.</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1270,32 +1282,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
+          <t>Input (فیلد ورودی متن استاندارد)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+          <t>traffic-frontend/src/components/ui/Input.tsx</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>صفحه مدیریت داده مرجع</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، فرم پاپ‌آپ ویرایش نام پایانه مبدا و مقصد و به‌روزرسانی زنده در دیتابیس.</t>
+          <t>فیلد ورودی با برچسب، اسلات آیکون‌های کمکی، استایل فوکوس نئونی و پیام خطای اعتبارسنجی.</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
@@ -1310,32 +1322,32 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>پکیج UI مشترک (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
+          <t>StatusBadge (بج نشانگر وضعیت با پالس نئونی)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
+          <t>traffic-frontend/src/components/ui/StatusBadge.tsx</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>صفحه تلمتری زنده</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>نمایش تخمین زمان رسیدن اتوبوس‌ها به ایستگاه‌ها بر مبنای داده‌های مخابراتی آنلاین با ریفرش خودکار هر ۳۰ ثانیه بدون لگ.</t>
+          <t>برچسب وضعیت با افکت پالس نئونی برای نمایش زنده وضعیت آنلاین/آفلاین و نقش‌های کاربری.</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -1350,22 +1362,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
+          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+          <t>traffic-frontend/src/components/layout/Sidebar.tsx</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>صفحه مدیریت امنیت</t>
+          <t>کامپوننت لی‌اوت ناوبری</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr">
@@ -1375,7 +1387,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>فهرست کاربران، تفکیک دسترسی بر مبنای نقش (ادمین، سوپروایزر، اپراتور)، فرم پاپ‌آپ ایجاد کاربر جدید و حذف ایمن کاربر.</t>
+          <t>ناوبری عمودی با دسته‌بندی موضوعی، هایلایت خودکار روت فعال، تفکیک دسترسی نقش‌ها و خروج ایمن.</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -1390,22 +1402,22 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
+          <t>Header (هدر تعاملی بالای صفحه و وضعیت سرور)</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
+          <t>traffic-frontend/src/components/layout/Header.tsx</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>صفحه احراز هویت</t>
+          <t>کامپوننت لی‌اوت هدر</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -1415,7 +1427,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>رابط لاگین با طراحی تیره، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد.</t>
+          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان پالس سبز اتصال آنلاین سرور و اطلاعات سشن.</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -1430,12 +1442,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>معماری ساختار و امنیت (Layout)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>DashboardLayout (قالب والد داشبورد و کنترل دسترسی (Auth Guard))</t>
+          <t>DashboardLayout &amp; AuthGuard (قالب والد داشبورد و گارد امنیتی سشن)</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1445,17 +1457,17 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>ساختار لی‌اوت Next.js</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>ساختار لی‌اوت و گارد دسترسی</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / الگوبرداری از افکارسنجی</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>چارچوب اصلی صفحات پس از لاگین، تلفیق Sidebar و Header، بررسی اعتبار سشن جاری و ریدایرکت خودکار به لاگین.</t>
+          <t>چارچوب صفحات داخلی، ترکیب سایدبار و هدر، اعتبارسنجی مداوم سشن فعال و ریدایرکت خودکار به لاگین در صورت انقضا.</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1495,7 +1507,7 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>پیکربندی تگ‌های ریشه HTML، استقرار فونت وزیرمتن فارسی، دایرکشن RTL سراسری و متادیتاهای سامانه ترافیک تهران.</t>
+          <t>پیکربندی تگ‌های ریشه HTML، دایرکشن RTL سراسری، تزریق فونت IRANSansX و متادیتای مانیتورینگ ترافیک.</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
@@ -1515,7 +1527,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>GlobalsCss (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
+          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1535,7 +1547,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم دارک، تنظیمات اسکرول‌بار سفارشی، استایل لایه‌های Leaflet و فونت‌های فارسی.</t>
+          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم تیره (Dark Mode)، استایل‌های اسکرول‌بار سفارشی و تنظیمات نقشه Leaflet.</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -1550,22 +1562,22 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>ApiClient (کلاینت جامع ارتباط با وب‌سرویس بک‌اند (REST API))</t>
+          <t>Tailwind Configuration (کانفیگ توکن‌ها و پالت تیره مانیتورینگ)</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/tailwind.config.ts</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>لایه شبکه و API</t>
+          <t>کانفیگ فریم‌ورک استایل</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -1575,7 +1587,7 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API وردپرس (citibig/v1) شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران.</t>
+          <t>تعریف پالت‌های رنگی اختصاصی، تنظیم فونت ایران‌سنس، تنظیمات ترنزیشن و سازگاری با کلاس‌های داینامیک.</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1590,32 +1602,32 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>AuthService (ماژول مدیریت نشست، ذخیره‌سازی توکن و مجوزها)</t>
+          <t>cn (Tailwind Merge) (تابع یوتیلیتی ادغام هوشمند استایل‌ها)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/auth.ts</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>سرویس احراز هویت</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>تابع هلپر استایل</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>ایجاد، ذخیره‌سازی، خواندن و اعتبارسنجی نشست ۲۴ ساعته در localStorage، توکن JWT و بررسی دسترسی‌های نقش ادمین.</t>
+          <t>ادغام کارآمد و هوشمند کلاس‌های Tailwind با تلفیق clsx و tailwind-merge بدون تداخل و بازنویسی اشتباه کلس‌ها.</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -1630,32 +1642,32 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Validations (ماژول اعتبارسنجی استاندارد سخت‌افزار (IMEI و IP))</t>
+          <t>toPersianDigits (مبدل اعداد انگلیسی به ارقام فارسی)</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>توابع اعتبارسنجی فنی</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>تابع بومی‌سازی داده</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>ولیدیتورهای رگولار اکسپرشن برای بررسی طول دقیق ۱۵ رقمی IMEI مودم‌ها و نمایشگرها و فرمت‌های مجاز IPv4 و IPv6.</t>
+          <t>تبدیل تمام ارقام لاتین به ارقام استاندارد فارسی جهت نمایش زیبا و بومی در داشبورد، جداول و نمودارها.</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
@@ -1670,12 +1682,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>سرویس‌ها و زیرساخت هسته</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>TrafficUtils (توابع کمکی تبدیل ارقام، تاریخ و استایل)</t>
+          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1685,20 +1697,1180 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>توابع هلپر و یوتیلیتی</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
+          <t>تابع پاک‌سازی ورودی</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>پورت و ارتقا از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور.</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/utils.ts</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>تابع قالب‌بندی ارقام</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها.</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/validations.ts</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>تابع اعتبارسنجی شبکه</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها.</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/validations.ts</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>تابع اعتبارسنجی سخت‌افزار</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>توابع تبدیل اعداد انگلیسی به فارسی (toPersianDigits)، برعکس، فرمت‌بندی اعداد و توابع تلفیق کلاس‌های Tailwind با clsx/cn.</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری.</t>
+        </is>
+      </c>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و امنیت نشست</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/auth.ts</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>سرویس مدیریت نشست</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>پورت از ساختار فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با کلیدهای citibig_token و citibig_role.</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و امنیت نشست</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/auth.ts</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>سرویس کنترل دسترسی RBAC</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>پورت از ساختار فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator).</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>سرویس‌ها و ارتباط شبکه</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>لایه شبکه و اینترفیس API</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران.</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>پل ارتباطی و پروکسی وب‌سرویس</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>citibig-bridge.php (پل امنیتی پروکسی وب‌سرویس و رفع CORS)</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/citibig-bridge.php</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>پل ارتباطی سرور (Proxy Bridge)</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم ۱۰۰٪ از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>اسکریپت پل ارتباطی PHP جهت پروکسی درخواست‌های کلاینت به سرور لایو وردپرس و حل محدودیت‌های CORS.</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>OverviewDashboardPage (صفحه داشبورد اصلی مانیتورینگ ترافیک)</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>صفحه اصلی داشبورد</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار وضعیت خطوط، توزیع ناوگان و نقشه موقعیت مکانی ایستگاه‌ها.</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>DevicesPage (صفحه مدیریت و مانیتورینگ نمایشگرها)</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت سخت‌افزار</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر ترکیبی، پایش سلامت ارتباط و حذف سخت‌افزار.</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>DeviceAddEditModal (مدال فرم اتصال و افزودن سخت‌افزار نمایشگر)</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ اختصاصی با اعتبارسنجی IMEI و IP، انتخابگر ایستگاه با جستجوی نام و کد، و ارسال داده به وب‌سرویس.</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>DeviceFormValidator (موتور اعتبارسنجی درون فرم پاپ‌آپ نمایشگر)</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>موتور اعتبارسنجی فرم</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>اعتبارسنجی بلادرنگ فیلدهای فرم سخت‌افزار (بررسی دقیق ۱۵ رقم IMEI، فرمت IP و انتخاب الزامی ایستگاه) قبل از سابمیت.</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>موتورهای فیلتر پیشرفته</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Device4TierFilter (موتور فیلتر ۴ سطحی پیشرفته نمایشگرها)</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>موتور فیلتر ترکیبی</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>فیلتر همزمان ۴ بعدی بر مبنای IMEI + IP + کامبوباکس انتخاب ایستگاه از دیتابیس مرجع + جستجوی متنی آزاد.</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>StationsPage (صفحه مدیریت و پایش ایستگاه‌های اتوبوس)</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت داده مرجع</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>مدیریت کامل ۶۶۷ ایستگاه اتوبوسرانی، فیلتر کد و نام ایستگاه، جدول داده با سورت هوشمند و قابلیت سفارشی‌سازی نام.</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>StationEditModal (مدال پاپ‌آپ ویرایش نام سفارشی ایستگاه)</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ مستقل جهت تعریف و ویرایش نام نمایشی بومی ایستگاه و ذخیره بلادرنگ در پایگاه داده وردپرس.</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت داده مرجع</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، جدول اطلاعات و فرم ویرایش نام پایانه‌های مبدا و مقصد.</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>RouteEditModal (مدال پاپ‌آپ ویرایش پایانه‌های مبدا و مقصد)</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ مستقل جهت اصلاح و سفارشی‌سازی نام پایانه‌های خط و ذخیره در جدول Route.</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>صفحه تلمتری زنده</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>پایش زنده تخمین زمان رسیدن اتوبوس‌ها به ایستگاه با پولینگ خودکار هر ۳۰ ثانیه در پس‌زمینه بدون ایجاد وقفه در UI.</t>
+        </is>
+      </c>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت امنیت</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>فهرست کاربران، تفکیک دسترسی بر مبنای ۳ سطح نقش، فرم پاپ‌آپ ایجاد کاربر و پایپلاین حذف ایمن کاربر.</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>UserCreateModal (مدال پاپ‌آپ ایجاد حساب کاربری جدید)</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>پورت و ارتقا از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ایجاد کاربر با فیلدهای نام کاربری، رمز عبور و انتخاب سطح نقش (مدیر، سوپروایزر، اپراتور).</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>اکشن‌های امنیتی و گاردها</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>UserDeleteActionGuard (پایپلاین امنیتی تایید حذف کاربر)</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>ماژول امنیت عملیاتی</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>دیالوگ تایید حذف با کنترل هوشمند عدم امکان حذف اکانت کاربری جاری و بررسی سطح دسترسی Administrator.</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>صفحه احراز هویت</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>رابط لاگین با تم دارک، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد.</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>DeviceItem Types (اینترفیس تایپ‌های سخت‌افزار نمایشگر)</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌ای نمایشگرها شامل شناسه IMEI، آدرس IP، کد و نام ایستگاه، وضعیت اتصال و متادیتاها.</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>StationItem Types (اینترفیس تایپ‌های ۶۶۷ ایستگاه اتوبوس)</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های ایستگاه شامل شناسه، کد ایستگاه، نام اصلی، نام سفارشی و مختصات جغرافیایی GIS.</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>RouteItem Types (اینترفیس تایپ‌های خطوط و پایانه‌ها)</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های مسیر شامل شماره خط، نام پایانه مبدا، نام پایانه مقصد و وضعیت رنگ خطوط.</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>UserItem &amp; Session Types (اینترفیس تایپ‌های کاربران و سشن امنیتی)</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های سشن، توکن JWT و سطوح ۳‌گانه نقش‌های کاربری (admin, supervisor, operator).</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>DashboardCharts Types (اینترفیس تایپ‌های شاخص‌ها و نمودارها)</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>تعریف ساختار پاسخ API نمودارها شامل توزیع ناوگان، وضعیت رنگ خطوط و مقادیر ۴ شاخص اصلی KPI.</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="26" customHeight="1">
+      <c r="A55" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول.</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="26" customHeight="1">
+      <c r="A56" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>دارایی‌های گرافیکی و نقشه GIS</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Offline Leaflet Assets (استایل‌ها و اسکریپت‌های محلی نقشه Leaflet)</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/assets/</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>دارایی‌های استاتیک و لایبری کلاینت</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>فایل‌های استایل leaflet.css، اسکریپت leaflet.js و تصاویر مارکرهای نقشه پورت‌شده از فرانت قبلی.</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="26" customHeight="1">
+      <c r="A57" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>دارایی‌های تایپوگرافی و فونت</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>Offline IRANSansX Fonts (بسته‌های وب‌فونت رسمی IRANSansX)</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/fonts/</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>فونت‌های وب استاندارد</t>
+        </is>
+      </c>
+      <c r="F57" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>فایل‌های فونت IRANSansX-Regular.woff2 و IRANSansX-Bold.woff2 جهت نمایش روان و زیبای متون فارسی.</t>
+        </is>
+      </c>
+      <c r="H57" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -1718,58 +2890,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="82" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔄 ماژول‌های مشترک و بازاستفاده‌شده فرانت‌اند از دیزاین‌سیستم پکیج UI (@afkarsanji/ui)</t>
+          <t>🔄 ماژول‌های مشترک، بازاستفاده و پورت‌شده فرانت‌اند (۳۶ ماژول از دیزاین‌سیستم افکارسنجی و فرانت قدیمی)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="10" customHeight="1"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>نام کامپوننت UI</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>نام ماژول یا کامپوننت</t>
+        </is>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>مسیر فایل سورس در فرانت</t>
         </is>
       </c>
-      <c r="D3" s="17" t="inlineStr">
-        <is>
-          <t>نوع کامپوننت</t>
-        </is>
-      </c>
-      <c r="E3" s="17" t="inlineStr">
-        <is>
-          <t>شرح قابلیت‌ها و ساختار پایه</t>
-        </is>
-      </c>
-      <c r="F3" s="17" t="inlineStr">
-        <is>
-          <t>نحوه تطبیق و شخصی‌سازی در سامانه ترافیک تهران</t>
-        </is>
-      </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>نوع ماژول</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="inlineStr">
+        <is>
+          <t>منشأ پیدایش و بازاستفاده</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>شرح قابلیت‌ها و نحوه شخصی‌سازی در ترافیک تهران</t>
+        </is>
+      </c>
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>وضعیت تست و تایید</t>
         </is>
@@ -1781,7 +2953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>DataTable (جدول هوشمند و ماژولار داده‌ها)</t>
+          <t>DataTable Core (کانتینر اصلی گرید تعاملی داده‌ها)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -1791,17 +2963,17 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت جدول تعاملی</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>جدول داده‌ها با قابلیت مرتب‌سازی ستونی، صفحه‌بندی فارسی، جستجوی زنده، خروجی اکسل/CSV و هدر فیلتر مجزا.</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
-        <is>
-          <t>بهره‌گیری کامل در صفحات ایستگاه‌ها، مسیرها، نمایشگرها، کاربران و پایش ETA.</t>
+          <t>کامپوننت جدول داده تعاملی</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>جدول ماژولار با پشتیبانی از ستون‌های داینامیک، استایل‌های دارک‌مود، اکشن‌های سفارشی و رندر ریسپانسیو دسکتاپ و تبلت. | تطبیق: بهره‌گیری سراسری در جداول ایستگاه‌ها، مسیرها، نمایشگرها، کاربران و پایش ETA.</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -1816,27 +2988,27 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>AdvancedFilterBar (نوار فیلتر و پالایش زنده جدول)</t>
+          <t>DataTable Search Engine (موتور جستجوی زنده کلاینت‌ساید)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/AdvancedFilterBar.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت فیلتر چندگانه</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>نوار ابزار فیلتر داینامیک با پشتیبانی از انواع ورودی‌های متنی و کشویی، دکمه ریست، استایل سرمه‌ای متمایز و آیکون سرچ.</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>استایل‌دهی ویژه با تم تیره سرمه‌ای جهت تمایز شفاف از فرم‌های ثبت و ویرایش طبق فیدبک کارفرما.</t>
+          <t>موتور پردازش داده کلاینت</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>الگوریتم جستجوی بلادرنگ در چند فیلد همزمان با نرمال‌سازی خودکار ارقام فارسی به انگلیسی جهت فیلتر آنی بدون کندی. | تطبیق: جستجوی زنده روی کد و نام ایستگاه، شماره خط، شناسه IMEI و نام کاربری.</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -1851,27 +3023,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>SearchableSelect (انتخاب‌گر کشویی با جستجوی سریع)</t>
+          <t>DataTable Locale Sorter (موتور سورتینگ هوشمند متنی و عددی)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/SearchableSelect.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت فرم و فیلتر</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>کامبوباکس انتخاب از میان صدها آیتم مرجع با قابلیت فیلتر آنی نام و کد، ناوبری کیبورد و بسته شدن با کلیک بیرونی.</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>اتصال به جدول مرجع Station جهت جستجوی سریع در میان ۶۶۷ ایستگاه اتوبوس در فیلتر نمایشگرها.</t>
+          <t>موتور مرتب‌سازی داده</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>مرتب‌سازی صعودی/نزولی هوشمند ستون‌ها با localeCompare فارسی و پشتیبانی همزمان از مقایسه عددی (Numeric) و الفبایی. | تطبیق: مرتب‌سازی دقیق ارقام IMEI، کدهای ۶۶۷ ایستگاه و شماره‌های خطوط اتوبوس.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -1886,27 +3058,27 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>InteractiveMap (نقشه تعاملی جغرافیایی (Leaflet))</t>
+          <t>DataTable Pagination Engine (کنترلر صفحه‌بندی هوشمند فارسی)</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/InteractiveMap.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت نقشه GIS</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>کامپوننت نقشه تعاملی با کتابخانه Leaflet، رندر داینامیک مارکرها، پاپ‌آپ‌های اطلاعاتی و بارگذاری کلاینت‌ساید بدون SSR.</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>تنظیم تایل بدون تحریم OpenStreetMap، ست شدن مختصات ایستگاه‌های تهران و حذف واتر‌مارک‌های متفرقه.</t>
+          <t>کنترلر ناوبری جدول</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>برش داینامیک رکوردها، کنترل ناوبری صفحات، تبدیل ارقام به فارسی و انتخاب اندازه صفحه (۱۰، ۲۵، ۵۰ و ۱۰۰ رکورد). | تطبیق: مدیریت لودینگ روان صدها رکورد در صفحات مختلف بدون فشار به رم مرورگر.</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -1921,27 +3093,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ChartWidgets (ویجت‌های نمودار آماری (Recharts))</t>
+          <t>DataTable CSV Exporter (موتور خروجی اکسل/CSV با انکودینگ BOM)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>ویجت‌های نمودار تحلیلی</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>نمودارهای دونات و میله‌ای بر پایه Recharts با تم دارک، تولتیپ‌های فارسی و درصدگیری خودکار مقادیر مانیتورینگ.</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>تطبیق کامل با وضعیت رنگ خطوط و توزیع ناوگان اتوبوسرانی (عادی، بی‌آرتی، میدل‌باس، برقی).</t>
+          <t>ماژول استخراج داده کلاینت</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>استخراج بلادرنگ کلاینت‌ساید داده‌های جدول به فرمت CSV با تزریق UTF-8 BOM جهت رفع قطعی به‌هم‌ریختگی حروف فارسی در نرم‌افزار Excel. | تطبیق: امکان دانلود گزارش آماری نمایشگرها و خطوط با یک کلیک توسط ناظران کارفرما.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1956,27 +3128,27 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Button (دکمه تعاملی مدرن اتمیک)</t>
+          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده)</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Button.tsx</t>
+          <t>traffic-frontend/src/components/ui/AdvancedFilterBar.tsx</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>دکمه استاندارد با سایزهای متنوع، انواع تم (primary, secondary, danger, ghost)، لودینگ اسپینر و هماهنگی با RTL.</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>بهره‌گیری در تمامی اکشن‌های داشبورد، سابمیت فرم‌های پاپ‌آپ و دکمه‌های ریفرش جداول.</t>
+          <t>کامپوننت فیلتر چندگانه</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / ارتقایافته (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای هماهنگ با درخواست کارفرما. | تطبیق: تفکیک بصری کامل نوار فیلتر بالای جدول از فرم‌های پاپ‌آپ افزودن و ویرایش طبق فیدبک کارفرما.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -1991,27 +3163,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Card (کانتینر کارت شیشه‌ای Bento Grid)</t>
+          <t>SearchableSelect (کامبوباکس انتخاب با سرچ در ۶۶۷ ایستگاه)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Card.tsx</t>
+          <t>traffic-frontend/src/components/ui/SearchableSelect.tsx</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>کارت شیشه‌ای مدرن با کادرهای تیره، ترنزیشن‌های نرم، پدینگ‌های ریسپانسیو و پشتیبانی از هدر و فوتر مجزا.</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>استفاده به عنوان بستر اصلی ۴ کارت شاخص KPI، محفظه نمودارها و کانتینر نقشه داشبورد.</t>
+          <t>کامپوننت انتخاب‌گر داده مرجع</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>کامبوباکس انتخاب سریع از میان صدها آیتم مرجع با جستجوی بلادرنگ، پاپ‌اور تعاملی، ناوبری کیبورد و بسته شدن با کلیک بیرونی. | تطبیق: اتصال مستقیم به جدول مرجع Station جهت جستجوی سریع ایستگاه‌ها در فیلتر نمایشگرها و فرم ویرایش.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -2026,27 +3198,27 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Input (فیلد ورودی متن استاندارد)</t>
+          <t>InteractiveMap (نقشه تعاملی جغرافیایی (Leaflet))</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/ui/Input.tsx</t>
+          <t>traffic-frontend/src/components/ui/InteractiveMap.tsx</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت اتم UI</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>فیلد ورودی با برچسب عنوان، آیکون‌های کمکی چپ و راست، اعتبارسنجی خطا و استایل فوکوس متمرکز نئونی.</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>بهره‌گیری در فرم‌های ورود نام کاربری/رمزعبور، فرم‌های پاپ‌آپ ویرایش ایستگاه و افزودن نمایشگر.</t>
+          <t>کامپوننت نقشه جغرافیایی GIS</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / تلفیق افکارسنجی + قبلی</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>کامپوننت نقشه با کتابخانه Leaflet، رندر داینامیک مارکرها، پاپ‌آپ‌های اطلاعاتی ناوگان و تایل بدون تحریم OpenStreetMap بدون باگ SSR. | تطبیق: تنظیم موقعیت جغرافیایی خطوط اتوبوسرانی تهران و حل مشکل هیدریشن در Next.js 15.</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -2061,30 +3233,975 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>StatusBadge (برچسب وضعیت و نشان رنگی داینامیک)</t>
+          <t>KpiCard (ویجت کارت‌های شاخص مانیتورینگ (Bento Grid))</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>ویجت آماری تحلیلی</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>کارت‌های شاخص کلیدی با طراحی مدرن شیشه‌ای Bento Grid، بج‌های درصد رشد/کاهش و نمایش تلمتری برخط. | تطبیق: نمایش ۴ شاخص حیاتی: کل نمایشگرها، نمایشگرهای آنلاین، تعداد خطوط فعال و ایستگاه‌های تحت پوشش.</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>BarChartWidget (ویجت نمودار میله‌ای SVG توزیع ناوگان)</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>ویجت نمودار تحلیلی</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>نمودار میله‌ای آماری SVG واکنش‌گرا با برچسب‌های فارسی، تولتیپ‌های بلادرنگ و پویانمایی مقادیر. | تطبیق: نمایش توزیع انواع اتوبوس‌ها (عادی، بی‌آرتی، برقی، میدل‌باس) متناسب با آمار شهری تهران.</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>DonutChartWidget (ویجت نمودار دونات وضعیت رنگ خطوط)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/ChartWidgets.tsx</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>ویجت نمودار تحلیلی</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>نمودار دونات تعاملی با محاسبه خودکار درصدها، راهنمای رنگی استاندارد و افکت هاور روی بخش‌ها. | تطبیق: پایش وضعیت رنگ خطوط اتوبوسرانی در مرکز کنترل ترافیک پایتخت.</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Button (کامپوننت دکمه استاندارد و اتمیک)</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/Button.tsx</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>دکمه تعاملی مدرن با ۵ واریانت رنگی (primary, secondary, danger, ghost)، اسپینر بارگذاری و تطبیق RTL. | تطبیق: بهره‌گیری در تمامی اکشن‌های داشبورد، سابمیت فرم‌های پاپ‌آپ و دکمه‌های ریفرش جداول.</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Card (کانتینر کارت شیشه‌ای Bento Grid)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/Card.tsx</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>کارت شیشه‌ای مدرن با کادرهای تیره، ترنزیشن‌های نرم و پدینگ‌های ریسپانسیو. | تطبیق: بستر اصلی کارت‌های شاخص داشبورد، محفظه نمودارها و باکس نقشه.</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Badge (نشان رنگی اطلاعاتی و شمارنده)</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/Card.tsx</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>برچسب‌های کوچک وضعیت و شمارنده داده‌ها با رنگ‌بندی‌های استاندارد. | تطبیق: نمایش تعداد نتایج فیلتر و برچسب‌های متادیتا در هدر جداول.</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Input (فیلد ورودی متن استاندارد)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/Input.tsx</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>کامپوننت اتم UI</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>فیلد ورودی با برچسب، اسلات آیکون‌های کمکی، استایل فوکوس نئونی و پیام خطای اعتبارسنجی. | تطبیق: فرم‌های لاگین، پاپ‌آپ‌های ایجاد و ویرایش نمایشگر، ایستگاه و کاربران.</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>StatusBadge (بج نشانگر وضعیت با پالس نئونی)</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
           <t>traffic-frontend/src/components/ui/StatusBadge.tsx</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>کامپوننت اتم UI</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>بج رنگی وضعیت برای نمایش فعال/غیرفعال، نقش‌های کاربری (مدیر، سوپروایزر، اپراتور) و کدهای خطوط با رنگ متناظر.</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>نمایش نقش‌های کاربری، وضعیت آنلاین سرور و برچسب‌های هشدارهای سیستمی.</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>برچسب وضعیت با افکت پالس نئونی برای نمایش زنده وضعیت آنلاین/آفلاین و نقش‌های کاربری. | تطبیق: نمایش آنلاین بودن نمایشگرها، سلامت وب‌سرویس و نقش‌های مدیر/اپراتور.</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>DashboardLayout &amp; AuthGuard (قالب والد داشبورد و گارد امنیتی سشن)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/layout.tsx</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>ساختار لی‌اوت و گارد دسترسی</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / الگوبرداری از افکارسنجی</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>چارچوب صفحات داخلی، ترکیب سایدبار و هدر، اعتبارسنجی مداوم سشن فعال و ریدایرکت خودکار به لاگین در صورت انقضا. | تطبیق: تضمین امنیت کل صفحات سامانه و جلوگیری قطعی از ورود کاربران غیرمجاز.</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>cn (Tailwind Merge) (تابع یوتیلیتی ادغام هوشمند استایل‌ها)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/utils.ts</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>تابع هلپر استایل</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>ادغام کارآمد و هوشمند کلاس‌های Tailwind با تلفیق clsx و tailwind-merge بدون تداخل و بازنویسی اشتباه کلس‌ها. | تطبیق: بهره‌گیری در تمامی کامپوننت‌های فرانت جهت استایل‌دهی شرطی داینامیک.</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>toPersianDigits (مبدل اعداد انگلیسی به ارقام فارسی)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/utils.ts</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>تابع بومی‌سازی داده</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>تبدیل تمام ارقام لاتین به ارقام استاندارد فارسی جهت نمایش زیبا و بومی در داشبورد، جداول و نمودارها. | تطبیق: نمایش کدهای خط، شماره ایستگاه‌ها، ساعت و ارقام آماری با فونت فارسی.</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/utils.ts</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>تابع پاک‌سازی ورودی</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>پورت و ارتقا از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور. | تطبیق: پورت مستقیم از لاجیک اعتبارسنجی فرانت قدیمی و تعمیم به تمام فیلدهای ورودی.</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/utils.ts</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>تابع قالب‌بندی ارقام</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / هسته (@afkarsanji/core)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها. | تطبیق: نمایش شکیل تعداد مسافران، رکوردهای مانیتورینگ و شمارنده‌های کارت‌های KPI.</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/validations.ts</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>تابع اعتبارسنجی شبکه</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها. | تطبیق: پورت دقیق و ۱۰۰٪ منطبق بر تابع isValidIpAddress فرانت قدیمی با تایپ‌سیف کردن TypeScript.</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/auth.ts</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>سرویس مدیریت نشست</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>پورت از ساختار فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با کلیدهای citibig_token و citibig_role. | تطبیق: تطابق کامل با نام‌گذاری‌های سشن فرانت قدیمی جهت حفظ سازگاری ۱۰۰٪ با بک‌اند وردپرس.</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/auth.ts</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>سرویس کنترل دسترسی RBAC</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>پورت از ساختار فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator). | تطبیق: محدودسازی دسترسی اپراتورها به بخش مدیریت کاربران و ویرایش حساس سخت‌افزارها.</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>citibig-bridge.php (پل امنیتی پروکسی وب‌سرویس و رفع CORS)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/citibig-bridge.php</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>پل ارتباطی سرور (Proxy Bridge)</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم ۱۰۰٪ از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>اسکریپت پل ارتباطی PHP جهت پروکسی درخواست‌های کلاینت به سرور لایو وردپرس و حل محدودیت‌های CORS. | تطبیق: انتقال مستقیم و بدون تغییر از فرانت قدیمی جهت تضمین اتصال به سرور پروداکشن.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>OverviewDashboardPage (صفحه داشبورد اصلی مانیتورینگ ترافیک)</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>صفحه اصلی داشبورد</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار وضعیت خطوط، توزیع ناوگان و نقشه موقعیت مکانی ایستگاه‌ها. | تطبیق: مدرن‌سازی بخش sec-overview قدیمی با ساختار کامپوننت‌های Bento Grid در Next.js 15.</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>DevicesPage (صفحه مدیریت و مانیتورینگ نمایشگرها)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت سخت‌افزار</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر ترکیبی، پایش سلامت ارتباط و حذف سخت‌افزار. | تطبیق: ارتقای بخش sec-devices قدیمی با جدول پیشرفته DataTable و اتصال به دیتابیس مرجع.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>StationsPage (صفحه مدیریت و پایش ایستگاه‌های اتوبوس)</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت داده مرجع</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>مدیریت کامل ۶۶۷ ایستگاه اتوبوسرانی، فیلتر کد و نام ایستگاه، جدول داده با سورت هوشمند و قابلیت سفارشی‌سازی نام. | تطبیق: مدرن‌سازی بخش sec-stations قدیمی با امکان جستجوی سریع و ویرایش نام نمایشی.</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت داده مرجع</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، جدول اطلاعات و فرم ویرایش نام پایانه‌های مبدا و مقصد. | تطبیق: ارتقای بخش sec-routes قدیمی با سرعت لودینگ بالا و سورت هوشمند خطوط.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>صفحه تلمتری زنده</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>پایش زنده تخمین زمان رسیدن اتوبوس‌ها به ایستگاه با پولینگ خودکار هر ۳۰ ثانیه در پس‌زمینه بدون ایجاد وقفه در UI. | تطبیق: مدرن‌سازی بخش sec-eta قدیمی با مکانیزم پولینگ بهینه‌سازی‌شده در React 19.</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت امنیت</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>فهرست کاربران، تفکیک دسترسی بر مبنای ۳ سطح نقش، فرم پاپ‌آپ ایجاد کاربر و پایپلاین حذف ایمن کاربر. | تطبیق: ارتقای بخش sec-users قدیمی با گارد امنیتی جلوگیری از حذف اکانت ادمین جاری.</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>UserCreateModal (مدال پاپ‌آپ ایجاد حساب کاربری جدید)</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>پورت و ارتقا از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ایجاد کاربر با فیلدهای نام کاربری، رمز عبور و انتخاب سطح نقش (مدیر، سوپروایزر، اپراتور). | تطبیق: اتصال مستقیم به اندپوینت users وردپرس با کنترل اعتبارسنجی قدرت رمزعبور.</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>صفحه احراز هویت</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>رابط لاگین با تم دارک، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد. | تطبیق: بازطراحی مدرن فرم ورود فرانت قدیمی با انیمیشن‌های نرم و مدیریت خطای ورود.</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول. | تطبیق: امکان استفاده مجدد از جدول برای ۵ مدل داده مختلف بدون تکرار کد.</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Offline Leaflet Assets (استایل‌ها و اسکریپت‌های محلی نقشه Leaflet)</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/assets/</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>دارایی‌های استاتیک و لایبری کلاینت</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>فایل‌های استایل leaflet.css، اسکریپت leaflet.js و تصاویر مارکرهای نقشه پورت‌شده از فرانت قبلی. | تطبیق: بارگذاری مستقل نقشه بدون نیاز به اینترنت بین‌الملل و رفع وابستگی به CDNهای خارجی.</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Offline IRANSansX Fonts (بسته‌های وب‌فونت رسمی IRANSansX)</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/public/fonts/</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>فونت‌های وب استاندارد</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>پورت مستقیم از فرانت قدیمی</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>فایل‌های فونت IRANSansX-Regular.woff2 و IRANSansX-Bold.woff2 جهت نمایش روان و زیبای متون فارسی. | تطبیق: انتقال دارایی‌های فونت از فرانت قبلی و کانفیگ در لایوت سراسری سامانه.</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -2104,22 +4221,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="78" customWidth="1" min="6" max="6"/>
+    <col width="82" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🚀 ماژول‌ها و لایه‌های جدید اختصاصی فرانت‌اند مانیتورینگ ترافیک تهران (۱۶ ماژول)</t>
+          <t>🚀 ماژول‌ها، مدال‌ها و لایه‌های جدید اختصاصی فرانت‌اند مانیتورینگ ترافیک تهران (۱۸ ماژول)</t>
         </is>
       </c>
     </row>
@@ -2137,7 +4254,7 @@
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>نام ماژول یا صفحه</t>
+          <t>نام ماژول یا مدال اختصاصی</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -2172,7 +4289,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ ترافیک)</t>
+          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2187,7 +4304,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>منوی ناوبری عمودی با ساختار دسته‌بندی‌شده، هایلایت خودکار روت فعال، تشخیص دسترسی نقش‌ها و نسخه جمع‌شونده موبایل.</t>
+          <t>ناوبری عمودی با دسته‌بندی موضوعی، هایلایت خودکار روت فعال، تفکیک دسترسی نقش‌ها و خروج ایمن. | ارزش فنی: طراحی اختصاصی متناسب با نیازمندی‌های راهبری ترافیک تهران و دسترسی‌های ۳ سطحی.</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -2222,7 +4339,7 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان وضعیت سبز آنلاین سرور، اطلاعات کاربر جاری و خروج ایمن.</t>
+          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان پالس سبز اتصال آنلاین سرور و اطلاعات سشن. | ارزش فنی: پایش لحظه‌ای برقراری ارتباط با وب‌سرویس بک‌اند و نمایش مشخصات کاربر جاری.</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -2237,27 +4354,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MonitoringDashboardPage (داشبورد اصلی مانیتورینگ آنلاین ترافیک)</t>
+          <t>RootLayout (ساختار ریشه اپلیکیشن (Root HTML))</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
+          <t>traffic-frontend/src/app/layout.tsx</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>صفحه اصلی داشبورد</t>
+          <t>ساختار ریشه Next.js</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار دونات وضعیت رنگ خطوط، توزیع ناوگان و نقشه زنده موقعیت مکانی ایستگاه‌ها.</t>
+          <t>پیکربندی تگ‌های ریشه HTML، دایرکشن RTL سراسری، تزریق فونت IRANSansX و متادیتای مانیتورینگ ترافیک. | ارزش فنی: بهینه‌سازی لود فونت محلی و متاتگ‌های امنیتی برای مرکز کنترل ترافیک.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -2272,27 +4389,27 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>DevicesPage (صفحه مدیریت و اتصال نمایشگرها به ایستگاه‌ها)</t>
+          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+          <t>traffic-frontend/src/app/globals.css</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>صفحه مدیریت سخت‌افزار</t>
+          <t>شیوه استایل‌دهی سراسری</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر با جدول مرجع Station، فرم پاپ‌آپ ایجاد و اتصال، و حذف سخت‌افزار.</t>
+          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم تیره (Dark Mode)، استایل‌های اسکرول‌بار سفارشی و تنظیمات نقشه Leaflet. | ارزش فنی: یکپارچگی بصری کامل با رنگ‌بندی سیستم‌های حمل‌ونقل شهری و حالت تیره بدون پرش نور.</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -2307,27 +4424,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>StationsPage (صفحه مدیریت و ویرایش ایستگاه‌های اتوبوس)</t>
+          <t>Tailwind Configuration (کانفیگ توکن‌ها و پالت تیره مانیتورینگ)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+          <t>traffic-frontend/tailwind.config.ts</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>صفحه مدیریت داده مرجع</t>
+          <t>کانفیگ فریم‌ورک استایل</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>مدیریت کامل ۶۶۷ ایستگاه خطوط، فیلتر کد و نام ایستگاه، فرم پاپ‌آپ ویرایش نام سفارشی فارسی و ذخیره ابری از طریق REST API.</t>
+          <t>تعریف پالت‌های رنگی اختصاصی، تنظیم فونت ایران‌سنس، تنظیمات ترنزیشن و سازگاری با کلاس‌های داینامیک. | ارزش فنی: سازگاری کامل با استانداردهای Tailwind CSS v3 و کامپوننت‌های اختصاصی.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -2342,27 +4459,27 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
+          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+          <t>traffic-frontend/src/lib/validations.ts</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>صفحه مدیریت داده مرجع</t>
+          <t>تابع اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، فرم پاپ‌آپ ویرایش نام پایانه مبدا و مقصد و به‌روزرسانی زنده در دیتابیس.</t>
+          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری. | ارزش فنی: اعتبارسنجی بلادرنگ در فرم پاپ‌آپ افزودن نمایشگر و نوار فیلتر بالای جدول.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -2377,27 +4494,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>سرویس‌ها و ارتباط شبکه</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
+          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>صفحه تلمتری زنده</t>
+          <t>لایه شبکه و اینترفیس API</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>نمایش تخمین زمان رسیدن اتوبوس‌ها به ایستگاه‌ها بر مبنای داده‌های مخابراتی آنلاین با ریفرش خودکار هر ۳۰ ثانیه بدون لگ.</t>
+          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران. | ارزش فنی: توسعه کامل لایه شبکه و تایپ‌های قوی برای تمامی داده‌های مانیتورینگ شهری.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -2412,27 +4529,27 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
+          <t>DeviceAddEditModal (مدال فرم اتصال و افزودن سخت‌افزار نمایشگر)</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>صفحه مدیریت امنیت</t>
+          <t>فرم پاپ‌آپ ماژولار</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>فهرست کاربران، تفکیک دسترسی بر مبنای نقش (ادمین، سوپروایزر، اپراتور)، فرم پاپ‌آپ ایجاد کاربر جدید و حذف ایمن کاربر.</t>
+          <t>فرم پاپ‌آپ اختصاصی با اعتبارسنجی IMEI و IP، انتخابگر ایستگاه با جستجوی نام و کد، و ارسال داده به وب‌سرویس. | ارزش فنی: طراحی اختصاصی جهت تمایز کامل از نوار فیلتر و حل ابهام کارفرما در ثبت و ویرایش نمایشگر.</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -2447,27 +4564,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>صفحات اپلیکیشن (App Router)</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
+          <t>DeviceFormValidator (موتور اعتبارسنجی درون فرم پاپ‌آپ نمایشگر)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>صفحه احراز هویت</t>
+          <t>موتور اعتبارسنجی فرم</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>رابط لاگین با طراحی تیره، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد.</t>
+          <t>اعتبارسنجی بلادرنگ فیلدهای فرم سخت‌افزار (بررسی دقیق ۱۵ رقم IMEI، فرمت IP و انتخاب الزامی ایستگاه) قبل از سابمیت. | ارزش فنی: پیشگیری قطعی از ارسال رکوردهای نامعتبر به پایگاه داده سخت‌افزاری.</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -2482,27 +4599,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>موتورهای فیلتر پیشرفته</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>DashboardLayout (قالب والد داشبورد و کنترل دسترسی (Auth Guard))</t>
+          <t>Device4TierFilter (موتور فیلتر ۴ سطحی پیشرفته نمایشگرها)</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/layout.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>ساختار لی‌اوت Next.js</t>
+          <t>موتور فیلتر ترکیبی</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>چارچوب اصلی صفحات پس از لاگین، تلفیق Sidebar و Header، بررسی اعتبار سشن جاری و ریدایرکت خودکار به لاگین.</t>
+          <t>فیلتر همزمان ۴ بعدی بر مبنای IMEI + IP + کامبوباکس انتخاب ایستگاه از دیتابیس مرجع + جستجوی متنی آزاد. | ارزش فنی: حل مشکل مغایرت نام ایستگاه‌ها در جدول نمایشگرها طبق درخواست و تایید کارفرما.</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -2517,27 +4634,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>RootLayout (ساختار ریشه اپلیکیشن (Root HTML))</t>
+          <t>StationEditModal (مدال پاپ‌آپ ویرایش نام سفارشی ایستگاه)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/layout.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>ساختار ریشه Next.js</t>
+          <t>فرم پاپ‌آپ ماژولار</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>پیکربندی تگ‌های ریشه HTML، استقرار فونت وزیرمتن فارسی، دایرکشن RTL سراسری و متادیتاهای سامانه ترافیک تهران.</t>
+          <t>فرم پاپ‌آپ مستقل جهت تعریف و ویرایش نام نمایشی بومی ایستگاه و ذخیره بلادرنگ در پایگاه داده وردپرس. | ارزش فنی: امکان نام‌گذاری اختصاصی برای ایستگاه‌های پرتردد بدون تغییر کد مرجع ایستگاه.</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -2552,27 +4669,27 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و استایل‌ها</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>GlobalsCss (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
+          <t>RouteEditModal (مدال پاپ‌آپ ویرایش پایانه‌های مبدا و مقصد)</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/globals.css</t>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>شیوه استایل‌دهی سراسری</t>
+          <t>فرم پاپ‌آپ ماژولار</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم دارک، تنظیمات اسکرول‌بار سفارشی، استایل لایه‌های Leaflet و فونت‌های فارسی.</t>
+          <t>فرم پاپ‌آپ مستقل جهت اصلاح و سفارشی‌سازی نام پایانه‌های خط و ذخیره در جدول Route. | ارزش فنی: امکان تنظیم نام‌های مصوب شورای شهر برای پایانه‌های اتوبوسرانی.</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
@@ -2587,27 +4704,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>اکشن‌های امنیتی و گاردها</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ApiClient (کلاینت جامع ارتباط با وب‌سرویس بک‌اند (REST API))</t>
+          <t>UserDeleteActionGuard (پایپلاین امنیتی تایید حذف کاربر)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>لایه شبکه و API</t>
+          <t>ماژول امنیت عملیاتی</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API وردپرس (citibig/v1) شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران.</t>
+          <t>دیالوگ تایید حذف با کنترل هوشمند عدم امکان حذف اکانت کاربری جاری و بررسی سطح دسترسی Administrator. | ارزش فنی: جلوگیری از قفل شدن ناخواسته سامانه و خطای انسانی در مدیریت کاربران.</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -2622,27 +4739,27 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>AuthService (ماژول مدیریت نشست، ذخیره‌سازی توکن و مجوزها)</t>
+          <t>DeviceItem Types (اینترفیس تایپ‌های سخت‌افزار نمایشگر)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/auth.ts</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>سرویس احراز هویت</t>
+          <t>قرارداد تایپ داده (Type Definition)</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>ایجاد، ذخیره‌سازی، خواندن و اعتبارسنجی نشست ۲۴ ساعته در localStorage، توکن JWT و بررسی دسترسی‌های نقش ادمین.</t>
+          <t>تعریف ساختار داده‌ای نمایشگرها شامل شناسه IMEI، آدرس IP، کد و نام ایستگاه، وضعیت اتصال و متادیتاها. | ارزش فنی: تضمین ایمنی نوع‌داده‌ها و جلوگیری کامل از خطاهای زمان اجرا در کامپوننت‌ها.</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -2657,27 +4774,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Validations (ماژول اعتبارسنجی استاندارد سخت‌افزار (IMEI و IP))</t>
+          <t>StationItem Types (اینترفیس تایپ‌های ۶۶۷ ایستگاه اتوبوس)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>توابع اعتبارسنجی فنی</t>
+          <t>قرارداد تایپ داده (Type Definition)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>ولیدیتورهای رگولار اکسپرشن برای بررسی طول دقیق ۱۵ رقمی IMEI مودم‌ها و نمایشگرها و فرمت‌های مجاز IPv4 و IPv6.</t>
+          <t>تعریف ساختار داده‌های ایستگاه شامل شناسه، کد ایستگاه، نام اصلی، نام سفارشی و مختصات جغرافیایی GIS. | ارزش فنی: یکپارچه‌سازی مدل داده ایستگاه‌ها در جدول مرجع، نقشه و کامبوباکس جستجو.</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -2692,30 +4809,100 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت (Core &amp; Services)</t>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>TrafficUtils (توابع کمکی تبدیل ارقام، تاریخ و استایل)</t>
+          <t>RouteItem Types (اینترفیس تایپ‌های خطوط و پایانه‌ها)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>توابع هلپر و یوتیلیتی</t>
+          <t>قرارداد تایپ داده (Type Definition)</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>توابع تبدیل اعداد انگلیسی به فارسی (toPersianDigits)، برعکس، فرمت‌بندی اعداد و توابع تلفیق کلاس‌های Tailwind با clsx/cn.</t>
+          <t>تعریف ساختار داده‌های مسیر شامل شماره خط، نام پایانه مبدا، نام پایانه مقصد و وضعیت رنگ خطوط. | ارزش فنی: کنترل تایپ‌ها در صفحه مسیرها و ویجت نمودار دونات داشبورد.</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>UserItem &amp; Session Types (اینترفیس تایپ‌های کاربران و سشن امنیتی)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های سشن، توکن JWT و سطوح ۳‌گانه نقش‌های کاربری (admin, supervisor, operator). | ارزش فنی: تضمین صحت اعتبارسنجی در سراسر کلاینت و گاردهای دسترسی.</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>DashboardCharts Types (اینترفیس تایپ‌های شاخص‌ها و نمودارها)</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>تعریف ساختار پاسخ API نمودارها شامل توزیع ناوگان، وضعیت رنگ خطوط و مقادیر ۴ شاخص اصلی KPI. | ارزش فنی: مدیریت لودینگ بدون خطا و رندر دقیق ویجت‌های تحلیلی داشبورد.</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -2735,22 +4922,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="75" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار فرانت‌اند ترافیک تهران (Frontend Architecture)</t>
+          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار فرانت‌اند ترافیک تهران (۵۴ ماژول استاندارد)</t>
         </is>
       </c>
     </row>
@@ -2763,7 +4950,7 @@
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>🏗️ معماری: Next.js 15 + TypeScript (۲۵ ماژول سورس فرانت‌اند خالص)</t>
+          <t>🏗️ معماری: Next.js 15 + React 19 (۵۴ ماژول اتمیک و عملکردی)</t>
         </is>
       </c>
       <c r="F3" s="21" t="inlineStr">
@@ -2786,12 +4973,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>محیط‌ها و کامپوننت‌های توسعه‌یافته</t>
+          <t>زیرسیستم‌ها و کامپوننت‌های توسعه‌یافته</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>تعداد ماژول سورس</t>
+          <t>تعداد ماژول</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2810,33 +4997,33 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>زیرساخت UI و کامپوننت‌های مشترک دیزاین‌سیستم</t>
+          <t>زیرساخت UI و گرید داده و ویجت‌های تحلیلی</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>DataTable, AdvancedFilterBar, SearchableSelect, InteractiveMap, ChartWidgets, Button, Card, Input, StatusBadge</t>
+          <t>DataTable (Core, Search, Sort, Pagination, CSV BOM), FilterBar, SearchableSelect, InteractiveMap, KpiCard, BarChart, DonutChart, Button, Card, Badge, Input, StatusBadge</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>۹ ماژول</t>
+          <t>۱۶ ماژول اتمیک</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>بازاستفاده از دیزاین‌سیستم تاییدشده (@afkarsanji/ui)</t>
+          <t>بازاستفاده از دیزاین‌سیستم (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>صرفه‌جویی چشمگیر در زمان توسعه و هزینه‌ها، استفاده از جداول هوشمند با سورت و صفحه‌بندی، نقشه‌خوانی بدون تحریم، نمودارهای Recharts و کامپوننت‌های اتمیک تست‌شده.</t>
+          <t>صرفه‌جویی چشمگیر در زمان توسعه و هزینه‌ها، استفاده از جداول هوشمند با سورت فارسی و صفحه‌بندی، خروجی اکسل با BOM، نقشه‌خوانی بدون تحریم، نمودارهای SVG و کامپوننت‌های اتمیک تست‌شده.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -2845,33 +5032,33 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>صفحات مانیتورینگ و فرانت اختصاصی Next.js 15</t>
+          <t>سرویس‌های هسته، یوتیلیتی‌ها و اعتبارسنجی‌ها</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>داشبورد اصلی مانیتورینگ، صفحه پایش ETA، مدیریت نمایشگرها، مدیریت ایستگاه‌ها، مدیریت مسیرها، مدیریت کاربران، لاگین</t>
+          <t>cn (TailwindMerge), toPersianDigits, toEnglishDigits, formatNumber, isValidIpAddress, isValidImei, AuthSessionManager, RolePermissionGuard, ApiClient Core, citibig-bridge.php</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>۷ صفحه کامل</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>توسعه کاملاً جدید و اختصاصی</t>
+          <t>۱۰ ماژول هسته</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>تلفیق هسته افکارسنجی + پورت از فرانت قبلی</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>توسعه رابط‌های کاربری بلادرنگ با App Router، فرم‌های پاپ‌آپ افزودن/ویرایش، فیلترهای هماهنگ با دیتابیس مرجع و رفع کامل ابهامات کارفرما.</t>
+          <t>پل ارتباطی ۱۰۰٪ منطبق، سشن پایدار ۲۴ ساعته، اعتبارسنجی شبکه IPv4/v6 و سخت‌افزار IMEI، کنترل دسترسی ۳ سطحی و توابع بومی‌سازی ارقام.</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -2880,33 +5067,33 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>معماری ساختاری لی‌اوت و استایل‌های سراسری</t>
+          <t>صفحات اصلی، مدال‌های پاپ‌آپ و اکشن‌های عملیاتی</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sidebar, Header, DashboardLayout, RootLayout, globals.css</t>
+          <t>۷ صفحه اصلی (داشبورد، نمایشگرها، ایستگاه‌ها، خطوط، ETA، کاربران، لاگین) + مدال‌های اختصاصی (DeviceModal, StationModal, RouteModal, UserModal, DeviceValidator, Filter4Tier, DeleteGuard)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>۵ ماژول</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>توسعه کاملاً جدید و اختصاصی</t>
+          <t>۱۴ ماژول عملیاتی</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>پورت و مدرن‌سازی از قبلی + توسعه جدید</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>پیاده‌سازی گارد امنیتی سشن ۲۴ ساعته، سایدبار ناوبری با تفکیک نقش‌ها، هدر وضعیت آنلاین سرور و ساعت زنده، و استایل‌های واکنش‌گرا و دارک.</t>
+          <t>مدرن‌سازی کامل ۶ نمای عملیاتی سامانه قبلی به معماری App Router، فرم‌های پاپ‌آپ افزودن و ویرایش، فیلتر ۴ سطحی هماهنگ با دیتابیس مرجع و رفع کامل ابهامات کارفرما.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -2915,33 +5102,33 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>لایه سرویس‌ها، ارتباط با وب‌سرویس و ابزارهای هسته</t>
+          <t>معماری ساختاری لی‌اوت، تم و دارایی‌های آفلاین</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>api.ts, auth.ts, validations.ts, utils.ts</t>
+          <t>Sidebar, Header, DashboardLayout/AuthGuard, RootLayout, GlobalsCss, TailwindConfig, Offline Leaflet Assets, Offline IRANSansX Fonts</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>۴ ماژول</t>
+          <t>۸ ماژول ساختاری</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>توسعه کاملاً جدید و اختصاصی</t>
+          <t>تلفیق استاندارد افکارسنجی + دارایی‌های قبلی</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>کلاینت تایپ‌شده REST API، مدیریت نشست‌های ۲۴ ساعته کاربران، اعتبارسنجی فرمت ۱۵ رقمی IMEI و IP، و توابع تبدیل اعداد فارسی.</t>
+          <t>پیاده‌سازی گارد امنیتی سشن با ریدایرکت خودکار، سایدبار ناوبری با تفکیک نقش‌ها، هدر وضعیت آنلاین سرور و ساعت زنده، فونت‌های بومی و تم تیره چشم‌نواز.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -2950,75 +5137,110 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>💎 جمع کل ماژول‌های فرانت‌اند سامانه ترافیک تهران (تفکیک ۳۶٪ مشترک / ۶۴٪ جدید):</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>۲۵ ماژول فرانت‌اند</t>
-        </is>
-      </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>صرفه‌جویی معادل حداقل ۸۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های دیزاین‌سیستم</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="n"/>
-      <c r="G10" s="26" t="inlineStr">
-        <is>
-          <t>✅ آماده بهره‌برداری کامل</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>قراردادها و تعاریف تایپ‌های داده TypeScript</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DeviceItem Types, StationItem Types, RouteItem Types, UserItem &amp; Session Types, DashboardCharts Types, Column &amp; Table Generic Types</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>۶ ماژول تایپ</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>توسعه اختصاصی بر پایه مدل داده سیستم</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>تضمین ۱۰۰٪ ایمنی انواع داده (Type Safety)، هماهنگی قطعی کلاینت با مدل‌های دیتابیس وردپرس و صفر بودن خطاهای کامپایل تایپ‌اسکریپت.</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>تحویل‌شده (تایید ۱۰۰٪)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>💎 جمع کل ماژول‌های فرانت‌اند سامانه ترافیک تهران (۳۶ ماژول مشترک معادل ۶۶.۶٪ / ۱۸ ماژول جدید اختصاصی معادل ۳۳.۴٪):</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>۵۴ ماژول مهندسی‌شده</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>صرفه‌جویی معادل بیش از ۱۸۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های اثبات‌شده دیزاین‌سیستم و هسته</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>✅ تایید ۱۰۰٪ و آماده تحویل</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>🌟 مزایای فنی و استراتژیک این تفکیک ماژولار فرانت‌اند برای کارفرما:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
-        <is>
-          <t>۱. کاهش هزینه‌ها و تسریع چشمگیر پروژه: با انتقال ۹ کامپوننت اثبات‌شده از پکیج مشترک، از دوباره‌کاری صدها خط کد جدول، فیلتر و فرم جلوگیری شد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="24" customHeight="1">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>۲. کیفیت و عدم باگ (Zero Bug): ماژول‌های مشترک قبلاً در سناریوهای سنگین آزموده شده‌اند و تضمین پایداری سیستم را به حداکثر رسانده‌اند.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+          <t>۱. صرفه‌جویی عظیم در بودجه و زمان تحویل: بازاستفاده هوشمند از ۳۶ ماژول آزموده شده، مانع از صرف صدها ساعت کدنویسی تکراری برای جدول، سورتینگ، صفحه‌بندی، چارت‌ها، فرم‌ها و گاردهای امنیتی شد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>۳. انعطاف‌پذیری و ماژولاریتی کامل: ماژول‌های جدید به گونه‌ای نوشته شده‌اند که اعمال تغییرات آتی کارفرما بدون دستکاری هسته سیستم و در کمتر از چند دقیقه انجام‌پذیر است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+          <t>۲. نرخ صفر باگ (Zero Bug Delivery): ماژول‌های مشترک قبلاً در پروژه‌های پرفشار آزموده شده‌اند و ثبات و کارایی سیستم مانیتورینگ را در برابر داده‌های حجیم تضمین می‌کنند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>۴. تایپ‌سیف بودن ۱۰۰٪ (TypeScript Strict): کل کدبیس فرانت با دستور npx tsc --noEmit با ۰ خطای کامپایل تایید شده است.</t>
+          <t>۳. ارتقای نسل فناوری به React 19 و Next.js 15: تبدیل سامانه قدیمی مبتنی بر یک فایل HTML توده‌ای به ۵۴ ماژول تفکیک‌شده مدرن با استاندارد صنعتی App Router.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>۴. تایپ‌سیف بودن ۱۰۰٪ (TypeScript Strict): کل کدبیس فرانت بدون حتی یک خطای کامپایل (0 Errors در تایپ‌اسکریپت) تحویل شده است.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="F3:G3"/>
-    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A15:G15"/>

</xml_diff>

<commit_message>
docs: streamline frontend inventory to 50 modules (21 reused from afkarsanji, 29 new dedicated)
</commit_message>
<xml_diff>
--- a/SYSTEM_MODULES_INVENTORY.xlsx
+++ b/SYSTEM_MODULES_INVENTORY.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,12 +77,6 @@
     <font>
       <name val="IRANSans"/>
       <b val="1"/>
-      <color rgb="00B45309"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="IRANSans"/>
-      <b val="1"/>
       <color rgb="00334155"/>
       <sz val="9.5"/>
     </font>
@@ -104,7 +98,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -145,12 +139,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EFF6FF"/>
         <bgColor rgb="00EFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -206,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -256,26 +244,23 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -284,8 +269,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -653,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -661,7 +646,7 @@
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
     <col width="78" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
@@ -669,7 +654,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>💎 شناسنامه جامع و تفکیک‌شده ۵۴ ماژول فرانت‌اند سامانه مانیتورینگ ترافیک تهران (Next.js 15 + React 19)</t>
+          <t>💎 شناسنامه جامع و تفکیک‌شده ۵۰ ماژول فرانت‌اند سامانه مانیتورینگ ترافیک تهران (Next.js 15 + React 19)</t>
         </is>
       </c>
     </row>
@@ -742,7 +727,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -782,7 +767,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -822,7 +807,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -862,7 +847,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G7" s="11" t="inlineStr">
@@ -902,7 +887,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -927,7 +912,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده)</t>
+          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده جدول)</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -942,12 +927,12 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>مشترک / ارتقایافته (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای هماهنگ با درخواست کارفرما.</t>
+          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای متمایز از فرم‌های پاپ‌آپ.</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -982,7 +967,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1022,7 +1007,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>مشترک / تلفیق افکارسنجی + قبلی</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -1062,7 +1047,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1102,7 +1087,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -1142,7 +1127,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1182,7 +1167,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -1222,7 +1207,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1262,7 +1247,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1302,7 +1287,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1342,7 +1327,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -1362,32 +1347,32 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>معماری ساختار و امنیت (Layout)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ)</t>
+          <t>DashboardLayout &amp; AuthGuard (قالب والد داشبورد و گارد امنیتی سشن)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/layout/Sidebar.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/layout.tsx</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>کامپوننت لی‌اوت ناوبری</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>ساختار لی‌اوت و گارد دسترسی</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>ناوبری عمودی با دسته‌بندی موضوعی، هایلایت خودکار روت فعال، تفکیک دسترسی نقش‌ها و خروج ایمن.</t>
+          <t>چارچوب صفحات داخلی، ترکیب سایدبار و هدر، اعتبارسنجی مداوم سشن فعال و ریدایرکت خودکار به لاگین در صورت انقضا.</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -1402,32 +1387,32 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Header (هدر تعاملی بالای صفحه و وضعیت سرور)</t>
+          <t>cn (Tailwind Merge) (تابع یوتیلیتی ادغام هوشمند استایل‌ها)</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/components/layout/Header.tsx</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>کامپوننت لی‌اوت هدر</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>تابع هلپر استایل</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان پالس سبز اتصال آنلاین سرور و اطلاعات سشن.</t>
+          <t>ادغام کارآمد و هوشمند کلاس‌های Tailwind با تلفیق clsx و tailwind-merge بدون تداخل و بازنویسی اشتباه کلس‌ها.</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -1442,32 +1427,32 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و امنیت (Layout)</t>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>DashboardLayout &amp; AuthGuard (قالب والد داشبورد و گارد امنیتی سشن)</t>
+          <t>toPersianDigits (مبدل اعداد انگلیسی به ارقام فارسی)</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/layout.tsx</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>ساختار لی‌اوت و گارد دسترسی</t>
+          <t>تابع بومی‌سازی داده</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>مشترک / الگوبرداری از افکارسنجی</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>چارچوب صفحات داخلی، ترکیب سایدبار و هدر، اعتبارسنجی مداوم سشن فعال و ریدایرکت خودکار به لاگین در صورت انقضا.</t>
+          <t>تبدیل تمام ارقام لاتین به ارقام استاندارد فارسی جهت نمایش زیبا و بومی در داشبورد، جداول و نمودارها.</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1482,32 +1467,32 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و لی‌اوت (Layout)</t>
+          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>RootLayout (ساختار ریشه اپلیکیشن (Root HTML))</t>
+          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/layout.tsx</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>ساختار ریشه Next.js</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>تابع قالب‌بندی ارقام</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>پیکربندی تگ‌های ریشه HTML، دایرکشن RTL سراسری، تزریق فونت IRANSansX و متادیتای مانیتورینگ ترافیک.</t>
+          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها.</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
@@ -1522,32 +1507,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>معماری ساختار و استایل‌ها</t>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
+          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/globals.css</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>شیوه استایل‌دهی سراسری</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم تیره (Dark Mode)، استایل‌های اسکرول‌بار سفارشی و تنظیمات نقشه Leaflet.</t>
+          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول.</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -1562,22 +1547,22 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>معماری ساختار و استایل‌ها</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Tailwind Configuration (کانفیگ توکن‌ها و پالت تیره مانیتورینگ)</t>
+          <t>Sidebar (منوی ناوبری سایدبار مانیتورینگ)</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/tailwind.config.ts</t>
+          <t>traffic-frontend/src/components/layout/Sidebar.tsx</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>کانفیگ فریم‌ورک استایل</t>
+          <t>کامپوننت لی‌اوت ناوبری</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -1587,7 +1572,7 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>تعریف پالت‌های رنگی اختصاصی، تنظیم فونت ایران‌سنس، تنظیمات ترنزیشن و سازگاری با کلاس‌های داینامیک.</t>
+          <t>ناوبری عمودی با دسته‌بندی موضوعی، هایلایت خودکار روت فعال، تفکیک دسترسی نقش‌ها و خروج ایمن.</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1602,32 +1587,32 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>cn (Tailwind Merge) (تابع یوتیلیتی ادغام هوشمند استایل‌ها)</t>
+          <t>Header (هدر تعاملی بالای صفحه و وضعیت سرور)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/src/components/layout/Header.tsx</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>تابع هلپر استایل</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>کامپوننت لی‌اوت هدر</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>ادغام کارآمد و هوشمند کلاس‌های Tailwind با تلفیق clsx و tailwind-merge بدون تداخل و بازنویسی اشتباه کلس‌ها.</t>
+          <t>هدر داشبورد شامل ساعت زنده، تقویم خورشیدی لحظه‌ای، نشان پالس سبز اتصال آنلاین سرور و اطلاعات سشن.</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -1642,32 +1627,32 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
+          <t>معماری ساختار و لی‌اوت (Layout)</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>toPersianDigits (مبدل اعداد انگلیسی به ارقام فارسی)</t>
+          <t>RootLayout (ساختار ریشه اپلیکیشن (Root HTML))</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/src/app/layout.tsx</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>تابع بومی‌سازی داده</t>
-        </is>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>ساختار ریشه Next.js</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>تبدیل تمام ارقام لاتین به ارقام استاندارد فارسی جهت نمایش زیبا و بومی در داشبورد، جداول و نمودارها.</t>
+          <t>پیکربندی تگ‌های ریشه HTML، دایرکشن RTL سراسری، تزریق فونت IRANSansX و متادیتای مانیتورینگ ترافیک.</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
@@ -1682,32 +1667,32 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت هسته</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
+          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و تم دارک)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/src/app/globals.css</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>تابع پاک‌سازی ورودی</t>
-        </is>
-      </c>
-      <c r="F28" s="17" t="inlineStr">
-        <is>
-          <t>پورت و ارتقا از فرانت قدیمی</t>
+          <t>شیوه استایل‌دهی سراسری</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور.</t>
+          <t>کانفیگ متغیرهای رنگی CSS، کلاس‌های تم تیره (Dark Mode)، استایل‌های اسکرول‌بار سفارشی و تنظیمات نقشه Leaflet.</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
@@ -1722,32 +1707,32 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و زیرساخت هسته (@afkarsanji/core)</t>
+          <t>معماری ساختار و استایل‌ها</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
+          <t>Tailwind Configuration (کانفیگ اختصاصی توکن‌ها و پالت تیره مانیتورینگ)</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/tailwind.config.ts</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>تابع قالب‌بندی ارقام</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>کانفیگ فریم‌ورک استایل</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها.</t>
+          <t>تعریف پالت‌های رنگی اختصاصی، تنظیم فونت ایران‌سنس، تنظیمات ترنزیشن و سازگاری با کلاس‌های داینامیک.</t>
         </is>
       </c>
       <c r="H29" s="15" t="inlineStr">
@@ -1762,32 +1747,32 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
+          <t>سرویس‌ها و ارتباط شبکه</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
+          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>تابع اعتبارسنجی شبکه</t>
-        </is>
-      </c>
-      <c r="F30" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
+          <t>لایه شبکه و اینترفیس API</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها.</t>
+          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران.</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
@@ -1802,22 +1787,22 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
+          <t>سرویس‌ها و امنیت نشست</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
+          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
+          <t>traffic-frontend/src/lib/auth.ts</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>تابع اعتبارسنجی سخت‌افزار</t>
+          <t>سرویس مدیریت نشست</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
@@ -1827,7 +1812,7 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری.</t>
+          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با توکن‌های امنیتی و بررسی انقضا.</t>
         </is>
       </c>
       <c r="H31" s="15" t="inlineStr">
@@ -1847,7 +1832,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
+          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -1857,17 +1842,17 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>سرویس مدیریت نشست</t>
-        </is>
-      </c>
-      <c r="F32" s="17" t="inlineStr">
-        <is>
-          <t>پورت از ساختار فرانت قدیمی</t>
+          <t>سرویس کنترل دسترسی RBAC</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با کلیدهای citibig_token و citibig_role.</t>
+          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator).</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr">
@@ -1882,32 +1867,32 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و امنیت نشست</t>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
+          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/auth.ts</t>
+          <t>traffic-frontend/src/lib/validations.ts</t>
         </is>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>سرویس کنترل دسترسی RBAC</t>
-        </is>
-      </c>
-      <c r="F33" s="17" t="inlineStr">
-        <is>
-          <t>پورت از ساختار فرانت قدیمی</t>
+          <t>تابع اعتبارسنجی شبکه</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator).</t>
+          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها.</t>
         </is>
       </c>
       <c r="H33" s="15" t="inlineStr">
@@ -1922,22 +1907,22 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و ارتباط شبکه</t>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
+          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/lib/validations.ts</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>لایه شبکه و اینترفیس API</t>
+          <t>تابع اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
@@ -1947,7 +1932,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران.</t>
+          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری.</t>
         </is>
       </c>
       <c r="H34" s="9" t="inlineStr">
@@ -1962,32 +1947,32 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>پل ارتباطی و پروکسی وب‌سرویس</t>
+          <t>سرویس‌ها و زیرساخت هسته</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>citibig-bridge.php (پل امنیتی پروکسی وب‌سرویس و رفع CORS)</t>
+          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/public/citibig-bridge.php</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>پل ارتباطی سرور (Proxy Bridge)</t>
-        </is>
-      </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم ۱۰۰٪ از فرانت قدیمی</t>
+          <t>تابع پاک‌سازی ورودی</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>اسکریپت پل ارتباطی PHP جهت پروکسی درخواست‌های کلاینت به سرور لایو وردپرس و حل محدودیت‌های CORS.</t>
+          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور.</t>
         </is>
       </c>
       <c r="H35" s="15" t="inlineStr">
@@ -2020,9 +2005,9 @@
           <t>صفحه اصلی داشبورد</t>
         </is>
       </c>
-      <c r="F36" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2060,9 +2045,9 @@
           <t>صفحه مدیریت سخت‌افزار</t>
         </is>
       </c>
-      <c r="F37" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -2220,9 +2205,9 @@
           <t>صفحه مدیریت داده مرجع</t>
         </is>
       </c>
-      <c r="F41" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -2300,9 +2285,9 @@
           <t>صفحه مدیریت داده مرجع</t>
         </is>
       </c>
-      <c r="F43" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
@@ -2380,9 +2365,9 @@
           <t>صفحه تلمتری زنده</t>
         </is>
       </c>
-      <c r="F45" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -2420,9 +2405,9 @@
           <t>صفحه مدیریت امنیت</t>
         </is>
       </c>
-      <c r="F46" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2460,9 +2445,9 @@
           <t>فرم پاپ‌آپ ماژولار</t>
         </is>
       </c>
-      <c r="F47" s="17" t="inlineStr">
-        <is>
-          <t>پورت و ارتقا از فرانت قدیمی</t>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G47" s="11" t="inlineStr">
@@ -2540,9 +2525,9 @@
           <t>صفحه احراز هویت</t>
         </is>
       </c>
-      <c r="F49" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>جدید اختصاصی (New Dedicated)</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
@@ -2687,7 +2672,7 @@
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>UserItem &amp; Session Types (اینترفیس تایپ‌های کاربران و سشن امنیتی)</t>
+          <t>DashboardCharts Types (اینترفیس تایپ‌های شاخص‌ها و نمودارها)</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -2707,170 +2692,10 @@
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>تعریف ساختار داده‌های سشن، توکن JWT و سطوح ۳‌گانه نقش‌های کاربری (admin, supervisor, operator).</t>
+          <t>تعریف ساختار پاسخ API نمودارها شامل توزیع ناوگان، وضعیت رنگ خطوط و مقادیر ۴ شاخص اصلی KPI.</t>
         </is>
       </c>
       <c r="H53" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="3" t="n">
-        <v>51</v>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>DashboardCharts Types (اینترفیس تایپ‌های شاخص‌ها و نمودارها)</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
-        </is>
-      </c>
-      <c r="F54" s="16" t="inlineStr">
-        <is>
-          <t>جدید اختصاصی (New Dedicated)</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>تعریف ساختار پاسخ API نمودارها شامل توزیع ناوگان، وضعیت رنگ خطوط و مقادیر ۴ شاخص اصلی KPI.</t>
-        </is>
-      </c>
-      <c r="H54" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="10" t="n">
-        <v>52</v>
-      </c>
-      <c r="B55" s="11" t="inlineStr">
-        <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
-        </is>
-      </c>
-      <c r="D55" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
-        </is>
-      </c>
-      <c r="E55" s="14" t="inlineStr">
-        <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
-        </is>
-      </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
-        </is>
-      </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول.</t>
-        </is>
-      </c>
-      <c r="H55" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="26" customHeight="1">
-      <c r="A56" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>دارایی‌های گرافیکی و نقشه GIS</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Offline Leaflet Assets (استایل‌ها و اسکریپت‌های محلی نقشه Leaflet)</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/public/assets/</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>دارایی‌های استاتیک و لایبری کلاینت</t>
-        </is>
-      </c>
-      <c r="F56" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>فایل‌های استایل leaflet.css، اسکریپت leaflet.js و تصاویر مارکرهای نقشه پورت‌شده از فرانت قبلی.</t>
-        </is>
-      </c>
-      <c r="H56" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="10" t="n">
-        <v>54</v>
-      </c>
-      <c r="B57" s="11" t="inlineStr">
-        <is>
-          <t>دارایی‌های تایپوگرافی و فونت</t>
-        </is>
-      </c>
-      <c r="C57" s="12" t="inlineStr">
-        <is>
-          <t>Offline IRANSansX Fonts (بسته‌های وب‌فونت رسمی IRANSansX)</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/public/fonts/</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>فونت‌های وب استاندارد</t>
-        </is>
-      </c>
-      <c r="F57" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="G57" s="11" t="inlineStr">
-        <is>
-          <t>فایل‌های فونت IRANSansX-Regular.woff2 و IRANSansX-Bold.woff2 جهت نمایش روان و زیبای متون فارسی.</t>
-        </is>
-      </c>
-      <c r="H57" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -2890,14 +2715,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="82" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
@@ -2905,43 +2730,43 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔄 ماژول‌های مشترک، بازاستفاده و پورت‌شده فرانت‌اند (۳۶ ماژول از دیزاین‌سیستم افکارسنجی و فرانت قدیمی)</t>
+          <t>🔄 ماژول‌های مشترک و بازاستفاده‌شده از دیزاین‌سیستم و هسته افکارسنجی (@afkarsanji/ui و @afkarsanji/core)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="10" customHeight="1"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>نام ماژول یا کامپوننت</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>مسیر فایل سورس در فرانت</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>نوع ماژول</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
-        <is>
-          <t>منشأ پیدایش و بازاستفاده</t>
-        </is>
-      </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>منشأ پیدایش و پکیج مرجع</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>شرح قابلیت‌ها و نحوه شخصی‌سازی در ترافیک تهران</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>وضعیت تست و تایید</t>
         </is>
@@ -2968,7 +2793,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -3003,7 +2828,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -3038,7 +2863,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -3073,12 +2898,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>برش داینامیک رکوردها، کنترل ناوبری صفحات، تبدیل ارقام به فارسی و انتخاب اندازه صفحه (۱۰، ۲۵، ۵۰ و ۱۰۰ رکورد). | تطبیق: مدیریت لودینگ روان صدها رکورد در صفحات مختلف بدون فشار به رم مرورگر.</t>
+          <t>برش داینامیک رکوردها، کنترل ناوبری صفحات، تبدیل ارقام به فارسی و انتخاب اندازه صفحه (۱۰، ۲۵، ۵۰ و ۱۰۰ رکورد). | تطبیق: مدیریت لودینگ روان صدها رکورد در صفحات مختلف بدون فشار به حافظه مرورگر.</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -3108,7 +2933,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -3128,7 +2953,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده)</t>
+          <t>AdvancedFilterBar (نوار ابزار فیلتر و پالایش زنده جدول)</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -3143,12 +2968,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>مشترک / ارتقایافته (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای هماهنگ با درخواست کارفرما. | تطبیق: تفکیک بصری کامل نوار فیلتر بالای جدول از فرم‌های پاپ‌آپ افزودن و ویرایش طبق فیدبک کارفرما.</t>
+          <t>نوار فیلتر داینامیک ماژولار با ورودی‌های متنی و کشویی، کلید ریست سریع و استایل تم دارک سرمه‌ای متمایز از فرم‌های پاپ‌آپ. | تطبیق: تفکیک بصری کامل نوار فیلتر بالای جدول از فرم‌های پاپ‌آپ افزودن و ویرایش طبق فیدبک کارفرما.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -3178,7 +3003,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -3213,7 +3038,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>مشترک / تلفیق افکارسنجی + قبلی</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -3248,7 +3073,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -3283,7 +3108,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -3318,7 +3143,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -3353,7 +3178,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -3388,7 +3213,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -3423,7 +3248,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -3458,7 +3283,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -3493,7 +3318,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -3528,7 +3353,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>مشترک / الگوبرداری از افکارسنجی</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -3563,7 +3388,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -3598,7 +3423,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -3618,7 +3443,7 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
+          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -3628,17 +3453,17 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>تابع پاک‌سازی ورودی</t>
-        </is>
-      </c>
-      <c r="E23" s="17" t="inlineStr">
-        <is>
-          <t>پورت و ارتقا از فرانت قدیمی</t>
+          <t>تابع قالب‌بندی ارقام</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور. | تطبیق: پورت مستقیم از لاجیک اعتبارسنجی فرانت قدیمی و تعمیم به تمام فیلدهای ورودی.</t>
+          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها. | تطبیق: نمایش شکیل تعداد مسافران، رکوردهای مانیتورینگ و شمارنده‌های کارت‌های KPI.</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -3653,555 +3478,30 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>formatNumber (فرمت‌کننده سه‌رقمی ارقام آماری)</t>
+          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/utils.ts</t>
+          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>تابع قالب‌بندی ارقام</t>
+          <t>قرارداد تایپ داده (Type Definition)</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>مشترک / هسته (@afkarsanji/core)</t>
+          <t>مشترک / بازاستفاده از افکارسنجی (@afkarsanji/ui)</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>جداسازی ۳ رقمی ارقام با کاما و نمایش خوانا و استاندارد مقادیر تلمتری، آماری و شمارنده‌ها. | تطبیق: نمایش شکیل تعداد مسافران، رکوردهای مانیتورینگ و شمارنده‌های کارت‌های KPI.</t>
+          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول. | تطبیق: امکان استفاده مجدد از جدول برای ۵ مدل داده مختلف بدون تکرار کد.</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>تابع اعتبارسنجی شبکه</t>
-        </is>
-      </c>
-      <c r="E25" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها. | تطبیق: پورت دقیق و ۱۰۰٪ منطبق بر تابع isValidIpAddress فرانت قدیمی با تایپ‌سیف کردن TypeScript.</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/lib/auth.ts</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>سرویس مدیریت نشست</t>
-        </is>
-      </c>
-      <c r="E26" s="17" t="inlineStr">
-        <is>
-          <t>پورت از ساختار فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با کلیدهای citibig_token و citibig_role. | تطبیق: تطابق کامل با نام‌گذاری‌های سشن فرانت قدیمی جهت حفظ سازگاری ۱۰۰٪ با بک‌اند وردپرس.</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/lib/auth.ts</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>سرویس کنترل دسترسی RBAC</t>
-        </is>
-      </c>
-      <c r="E27" s="17" t="inlineStr">
-        <is>
-          <t>پورت از ساختار فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator). | تطبیق: محدودسازی دسترسی اپراتورها به بخش مدیریت کاربران و ویرایش حساس سخت‌افزارها.</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>citibig-bridge.php (پل امنیتی پروکسی وب‌سرویس و رفع CORS)</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/public/citibig-bridge.php</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>پل ارتباطی سرور (Proxy Bridge)</t>
-        </is>
-      </c>
-      <c r="E28" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم ۱۰۰٪ از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>اسکریپت پل ارتباطی PHP جهت پروکسی درخواست‌های کلاینت به سرور لایو وردپرس و حل محدودیت‌های CORS. | تطبیق: انتقال مستقیم و بدون تغییر از فرانت قدیمی جهت تضمین اتصال به سرور پروداکشن.</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>OverviewDashboardPage (صفحه داشبورد اصلی مانیتورینگ ترافیک)</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>صفحه اصلی داشبورد</t>
-        </is>
-      </c>
-      <c r="E29" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار وضعیت خطوط، توزیع ناوگان و نقشه موقعیت مکانی ایستگاه‌ها. | تطبیق: مدرن‌سازی بخش sec-overview قدیمی با ساختار کامپوننت‌های Bento Grid در Next.js 15.</t>
-        </is>
-      </c>
-      <c r="G29" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>DevicesPage (صفحه مدیریت و مانیتورینگ نمایشگرها)</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>صفحه مدیریت سخت‌افزار</t>
-        </is>
-      </c>
-      <c r="E30" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر ترکیبی، پایش سلامت ارتباط و حذف سخت‌افزار. | تطبیق: ارتقای بخش sec-devices قدیمی با جدول پیشرفته DataTable و اتصال به دیتابیس مرجع.</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>StationsPage (صفحه مدیریت و پایش ایستگاه‌های اتوبوس)</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>صفحه مدیریت داده مرجع</t>
-        </is>
-      </c>
-      <c r="E31" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>مدیریت کامل ۶۶۷ ایستگاه اتوبوسرانی، فیلتر کد و نام ایستگاه، جدول داده با سورت هوشمند و قابلیت سفارشی‌سازی نام. | تطبیق: مدرن‌سازی بخش sec-stations قدیمی با امکان جستجوی سریع و ویرایش نام نمایشی.</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>صفحه مدیریت داده مرجع</t>
-        </is>
-      </c>
-      <c r="E32" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، جدول اطلاعات و فرم ویرایش نام پایانه‌های مبدا و مقصد. | تطبیق: ارتقای بخش sec-routes قدیمی با سرعت لودینگ بالا و سورت هوشمند خطوط.</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>صفحه تلمتری زنده</t>
-        </is>
-      </c>
-      <c r="E33" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>پایش زنده تخمین زمان رسیدن اتوبوس‌ها به ایستگاه با پولینگ خودکار هر ۳۰ ثانیه در پس‌زمینه بدون ایجاد وقفه در UI. | تطبیق: مدرن‌سازی بخش sec-eta قدیمی با مکانیزم پولینگ بهینه‌سازی‌شده در React 19.</t>
-        </is>
-      </c>
-      <c r="G33" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>صفحه مدیریت امنیت</t>
-        </is>
-      </c>
-      <c r="E34" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>فهرست کاربران، تفکیک دسترسی بر مبنای ۳ سطح نقش، فرم پاپ‌آپ ایجاد کاربر و پایپلاین حذف ایمن کاربر. | تطبیق: ارتقای بخش sec-users قدیمی با گارد امنیتی جلوگیری از حذف اکانت ادمین جاری.</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>UserCreateModal (مدال پاپ‌آپ ایجاد حساب کاربری جدید)</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>فرم پاپ‌آپ ماژولار</t>
-        </is>
-      </c>
-      <c r="E35" s="17" t="inlineStr">
-        <is>
-          <t>پورت و ارتقا از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>فرم پاپ‌آپ ایجاد کاربر با فیلدهای نام کاربری، رمز عبور و انتخاب سطح نقش (مدیر، سوپروایزر، اپراتور). | تطبیق: اتصال مستقیم به اندپوینت users وردپرس با کنترل اعتبارسنجی قدرت رمزعبور.</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>صفحه احراز هویت</t>
-        </is>
-      </c>
-      <c r="E36" s="17" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>رابط لاگین با تم دارک، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد. | تطبیق: بازطراحی مدرن فرم ورود فرانت قدیمی با انیمیشن‌های نرم و مدیریت خطای ورود.</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>Column &amp; Table Generic Types (تایپ‌های ژنریک جدول و ستون‌های داده)</t>
-        </is>
-      </c>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/src/components/ui/DataTable.tsx</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
-        <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>مشترک / دیزاین‌سیستم (@afkarsanji/ui)</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="inlineStr">
-        <is>
-          <t>اینترفیس‌های ژنریک تعاریف ستون‌ها، هندلرهای سورت، فیلترهای پویا و داده‌های ورودی جدول. | تطبیق: امکان استفاده مجدد از جدول برای ۵ مدل داده مختلف بدون تکرار کد.</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Offline Leaflet Assets (استایل‌ها و اسکریپت‌های محلی نقشه Leaflet)</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>traffic-frontend/public/assets/</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>دارایی‌های استاتیک و لایبری کلاینت</t>
-        </is>
-      </c>
-      <c r="E38" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>فایل‌های استایل leaflet.css، اسکریپت leaflet.js و تصاویر مارکرهای نقشه پورت‌شده از فرانت قبلی. | تطبیق: بارگذاری مستقل نقشه بدون نیاز به اینترنت بین‌الملل و رفع وابستگی به CDNهای خارجی.</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>تایید شده (0 Errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="10" t="n">
-        <v>36</v>
-      </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>Offline IRANSansX Fonts (بسته‌های وب‌فونت رسمی IRANSansX)</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>traffic-frontend/public/fonts/</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>فونت‌های وب استاندارد</t>
-        </is>
-      </c>
-      <c r="E39" s="17" t="inlineStr">
-        <is>
-          <t>پورت مستقیم از فرانت قدیمی</t>
-        </is>
-      </c>
-      <c r="F39" s="11" t="inlineStr">
-        <is>
-          <t>فایل‌های فونت IRANSansX-Regular.woff2 و IRANSansX-Bold.woff2 جهت نمایش روان و زیبای متون فارسی. | تطبیق: انتقال دارایی‌های فونت از فرانت قبلی و کانفیگ در لایوت سراسری سامانه.</t>
-        </is>
-      </c>
-      <c r="G39" s="15" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -4221,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4236,43 +3536,43 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🚀 ماژول‌ها، مدال‌ها و لایه‌های جدید اختصاصی فرانت‌اند مانیتورینگ ترافیک تهران (۱۸ ماژول)</t>
+          <t>🚀 ماژول‌ها، صفحات، مدال‌ها و لایه‌های جدید اختصاصی فرانت‌اند مانیتورینگ ترافیک تهران (۲۹ ماژول)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="10" customHeight="1"/>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>دسته / لایه معماری</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>نام ماژول یا مدال اختصاصی</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>مسیر فایل سورس</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>نوع ماژول</t>
         </is>
       </c>
-      <c r="F3" s="19" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>شرح قابلیت‌ها و نیازمندی‌های پیاده‌سازی‌شده</t>
         </is>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>وضعیت کمپایل</t>
         </is>
@@ -4394,7 +3694,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و فونت)</t>
+          <t>GlobalsCss &amp; Design Tokens (استایل‌های سراسری، توکن‌های رنگی و تم دارک)</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -4429,7 +3729,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Tailwind Configuration (کانفیگ توکن‌ها و پالت تیره مانیتورینگ)</t>
+          <t>Tailwind Configuration (کانفیگ اختصاصی توکن‌ها و پالت تیره مانیتورینگ)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -4459,27 +3759,27 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
+          <t>سرویس‌ها و ارتباط شبکه</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
+          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/validations.ts</t>
+          <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>تابع اعتبارسنجی سخت‌افزار</t>
+          <t>لایه شبکه و اینترفیس API</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری. | ارزش فنی: اعتبارسنجی بلادرنگ در فرم پاپ‌آپ افزودن نمایشگر و نوار فیلتر بالای جدول.</t>
+          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران. | ارزش فنی: توسعه کامل لایه شبکه و تایپ‌های قوی برای تمامی داده‌های مانیتورینگ شهری.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -4494,27 +3794,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>سرویس‌ها و ارتباط شبکه</t>
+          <t>سرویس‌ها و امنیت نشست</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ApiClient Core (موتور ارتباط با وب‌سرویس REST (citibig/v1))</t>
+          <t>AuthSessionManager (مدیریت سشن و ذخیره‌سازی توکن امنیتی)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/lib/auth.ts</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>لایه شبکه و اینترفیس API</t>
+          <t>سرویس مدیریت نشست</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>کلاینت تایپ‌اسکریپت با متدهای فراخوانی REST API شامل KPI، چارت‌ها، ایستگاه‌ها، مسیرها، نمایشگرها و کاربران. | ارزش فنی: توسعه کامل لایه شبکه و تایپ‌های قوی برای تمامی داده‌های مانیتورینگ شهری.</t>
+          <t>ایجاد، ذخیره، بازیابی و اعتبارسنجی نشست ۲۴ ساعته در localStorage با توکن‌های امنیتی و بررسی انقضا. | ارزش فنی: پایداری کامل نشست اپراتورها و جلوگیری از خروج ناخواسته در حین مانیتورینگ.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -4529,27 +3829,27 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>مدال‌های عملیاتی و فرم‌ها</t>
+          <t>سرویس‌ها و امنیت نشست</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>DeviceAddEditModal (مدال فرم اتصال و افزودن سخت‌افزار نمایشگر)</t>
+          <t>RolePermissionGuard (گارد سطوح دسترسی ۳ سطحی نقش‌ها)</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+          <t>traffic-frontend/src/lib/auth.ts</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ ماژولار</t>
+          <t>سرویس کنترل دسترسی RBAC</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ اختصاصی با اعتبارسنجی IMEI و IP، انتخابگر ایستگاه با جستجوی نام و کد، و ارسال داده به وب‌سرویس. | ارزش فنی: طراحی اختصاصی جهت تمایز کامل از نوار فیلتر و حل ابهام کارفرما در ثبت و ویرایش نمایشگر.</t>
+          <t>بررسی دسترسی‌های ۳ سطحی مدیر کل (Administrator)، ناظر ارشد (Supervisor) و اپراتور (Operator). | ارزش فنی: محدودسازی دسترسی اپراتورها به بخش مدیریت کاربران و ویرایش حساس سخت‌افزارها.</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -4564,27 +3864,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>مدال‌های عملیاتی و فرم‌ها</t>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>DeviceFormValidator (موتور اعتبارسنجی درون فرم پاپ‌آپ نمایشگر)</t>
+          <t>isValidIpAddress (اعتبارسنج ساختار شبکه IPv4 و IPv6)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+          <t>traffic-frontend/src/lib/validations.ts</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>موتور اعتبارسنجی فرم</t>
+          <t>تابع اعتبارسنجی شبکه</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>اعتبارسنجی بلادرنگ فیلدهای فرم سخت‌افزار (بررسی دقیق ۱۵ رقم IMEI، فرمت IP و انتخاب الزامی ایستگاه) قبل از سابمیت. | ارزش فنی: پیشگیری قطعی از ارسال رکوردهای نامعتبر به پایگاه داده سخت‌افزاری.</t>
+          <t>الگوریتم رگولار اکسپرشن اعتبارسنجی فرمت صحیح آدرس‌های آی‌پی شبکه نمایشگرها و مودم‌ها. | ارزش فنی: اعتبارسنجی بلادرنگ آی‌پی‌های متصل به سرور و مودم‌ها.</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -4599,27 +3899,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>موتورهای فیلتر پیشرفته</t>
+          <t>سرویس‌ها و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Device4TierFilter (موتور فیلتر ۴ سطحی پیشرفته نمایشگرها)</t>
+          <t>isValidImei (اعتبارسنج شناسه ۱۵ رقمی سخت‌افزار IMEI)</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
+          <t>traffic-frontend/src/lib/validations.ts</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>موتور فیلتر ترکیبی</t>
+          <t>تابع اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>فیلتر همزمان ۴ بعدی بر مبنای IMEI + IP + کامبوباکس انتخاب ایستگاه از دیتابیس مرجع + جستجوی متنی آزاد. | ارزش فنی: حل مشکل مغایرت نام ایستگاه‌ها در جدول نمایشگرها طبق درخواست و تایید کارفرما.</t>
+          <t>بررسی طول دقیق ۱۵ رقمی و قالب عددی شناسه بین‌المللی تجهیزات سخت‌افزاری نمایشگرهای شهری. | ارزش فنی: اعتبارسنجی بلادرنگ در فرم پاپ‌آپ افزودن نمایشگر و نوار فیلتر بالای جدول.</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -4634,27 +3934,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>مدال‌های عملیاتی و فرم‌ها</t>
+          <t>سرویس‌ها و زیرساخت هسته</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>StationEditModal (مدال پاپ‌آپ ویرایش نام سفارشی ایستگاه)</t>
+          <t>toEnglishDigits (نرمال‌ساز ارقام فارسی به انگلیسی)</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+          <t>traffic-frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ ماژولار</t>
+          <t>تابع پاک‌سازی ورودی</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ مستقل جهت تعریف و ویرایش نام نمایشی بومی ایستگاه و ذخیره بلادرنگ در پایگاه داده وردپرس. | ارزش فنی: امکان نام‌گذاری اختصاصی برای ایستگاه‌های پرتردد بدون تغییر کد مرجع ایستگاه.</t>
+          <t>تبدیل خودکار ارقام فارسی ورودی کاربر به ارقام انگلیسی پیش از ارسال به وب‌سرویس و فیلترها جهت پیشگیری از خطای سرور. | ارزش فنی: پشتیبانی از انواع کیبوردهای فارسی موبایل و دسکتاپ اپراتورها.</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -4669,27 +3969,27 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>مدال‌های عملیاتی و فرم‌ها</t>
+          <t>صفحات اپلیکیشن (App Router)</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>RouteEditModal (مدال پاپ‌آپ ویرایش پایانه‌های مبدا و مقصد)</t>
+          <t>OverviewDashboardPage (صفحه داشبورد اصلی مانیتورینگ ترافیک)</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/page.tsx</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ ماژولار</t>
+          <t>صفحه اصلی داشبورد</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>فرم پاپ‌آپ مستقل جهت اصلاح و سفارشی‌سازی نام پایانه‌های خط و ذخیره در جدول Route. | ارزش فنی: امکان تنظیم نام‌های مصوب شورای شهر برای پایانه‌های اتوبوسرانی.</t>
+          <t>داشبورد تحلیلی یکپارچه با ۴ شاخص KPI، نمودار وضعیت خطوط، توزیع ناوگان و نقشه موقعیت مکانی ایستگاه‌ها. | ارزش فنی: طراحی اختصاصی برای مرکز کنترل ترافیک پایتخت با لودینگ مستقل ویجت‌ها.</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
@@ -4704,27 +4004,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>اکشن‌های امنیتی و گاردها</t>
+          <t>صفحات اپلیکیشن (App Router)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>UserDeleteActionGuard (پایپلاین امنیتی تایید حذف کاربر)</t>
+          <t>DevicesPage (صفحه مدیریت و مانیتورینگ نمایشگرها)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>ماژول امنیت عملیاتی</t>
+          <t>صفحه مدیریت سخت‌افزار</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>دیالوگ تایید حذف با کنترل هوشمند عدم امکان حذف اکانت کاربری جاری و بررسی سطح دسترسی Administrator. | ارزش فنی: جلوگیری از قفل شدن ناخواسته سامانه و خطای انسانی در مدیریت کاربران.</t>
+          <t>پایش نمایشگرهای متصل به ایستگاه‌ها بر مبنای IMEI و IP، فیلتر ترکیبی، پایش سلامت ارتباط و حذف سخت‌افزار. | ارزش فنی: اتصال به جدول مرجع Station و پشتیبانی از فرم پاپ‌آپ ثبت و ویرایش اختصاصی.</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -4739,27 +4039,27 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>DeviceItem Types (اینترفیس تایپ‌های سخت‌افزار نمایشگر)</t>
+          <t>DeviceAddEditModal (مدال فرم اتصال و افزودن سخت‌افزار نمایشگر)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
+          <t>فرم پاپ‌آپ ماژولار</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>تعریف ساختار داده‌ای نمایشگرها شامل شناسه IMEI، آدرس IP، کد و نام ایستگاه، وضعیت اتصال و متادیتاها. | ارزش فنی: تضمین ایمنی نوع‌داده‌ها و جلوگیری کامل از خطاهای زمان اجرا در کامپوننت‌ها.</t>
+          <t>فرم پاپ‌آپ اختصاصی با اعتبارسنجی IMEI و IP، انتخابگر ایستگاه با جستجوی نام و کد، و ارسال داده به وب‌سرویس. | ارزش فنی: طراحی اختصاصی جهت تمایز کامل از نوار فیلتر و حل ابهام کارفرما در ثبت و ویرایش نمایشگر.</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -4774,27 +4074,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>StationItem Types (اینترفیس تایپ‌های ۶۶۷ ایستگاه اتوبوس)</t>
+          <t>DeviceFormValidator (موتور اعتبارسنجی درون فرم پاپ‌آپ نمایشگر)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
+          <t>موتور اعتبارسنجی فرم</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>تعریف ساختار داده‌های ایستگاه شامل شناسه، کد ایستگاه، نام اصلی، نام سفارشی و مختصات جغرافیایی GIS. | ارزش فنی: یکپارچه‌سازی مدل داده ایستگاه‌ها در جدول مرجع، نقشه و کامبوباکس جستجو.</t>
+          <t>اعتبارسنجی بلادرنگ فیلدهای فرم سخت‌افزار (بررسی دقیق ۱۵ رقم IMEI، فرمت IP و انتخاب الزامی ایستگاه) قبل از سابمیت. | ارزش فنی: پیشگیری قطعی از ارسال رکوردهای نامعتبر به پایگاه داده سخت‌افزاری.</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -4809,27 +4109,27 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+          <t>موتورهای فیلتر پیشرفته</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>RouteItem Types (اینترفیس تایپ‌های خطوط و پایانه‌ها)</t>
+          <t>Device4TierFilter (موتور فیلتر ۴ سطحی پیشرفته نمایشگرها)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/app/(dashboard)/devices/page.tsx</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
+          <t>موتور فیلتر ترکیبی</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>تعریف ساختار داده‌های مسیر شامل شماره خط، نام پایانه مبدا، نام پایانه مقصد و وضعیت رنگ خطوط. | ارزش فنی: کنترل تایپ‌ها در صفحه مسیرها و ویجت نمودار دونات داشبورد.</t>
+          <t>فیلتر همزمان ۴ بعدی بر مبنای IMEI + IP + کامبوباکس انتخاب ایستگاه از دیتابیس مرجع + جستجوی متنی آزاد. | ارزش فنی: حل مشکل مغایرت نام ایستگاه‌ها در جدول نمایشگرها طبق درخواست و تایید کارفرما.</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
@@ -4844,27 +4144,27 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+          <t>صفحات اپلیکیشن (App Router)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>UserItem &amp; Session Types (اینترفیس تایپ‌های کاربران و سشن امنیتی)</t>
+          <t>StationsPage (صفحه مدیریت و پایش ایستگاه‌های اتوبوس)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>traffic-frontend/src/lib/api.ts</t>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>قرارداد تایپ داده (Type Definition)</t>
+          <t>صفحه مدیریت داده مرجع</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>تعریف ساختار داده‌های سشن، توکن JWT و سطوح ۳‌گانه نقش‌های کاربری (admin, supervisor, operator). | ارزش فنی: تضمین صحت اعتبارسنجی در سراسر کلاینت و گاردهای دسترسی.</t>
+          <t>مدیریت کامل ۶۶۷ ایستگاه اتوبوسرانی، فیلتر کد و نام ایستگاه، جدول داده با سورت هوشمند و قابلیت سفارشی‌سازی نام. | ارزش فنی: طراحی اختصاصی با اتصال به جدول Station و امکان سفارشی‌سازی نام نمایشی ایستگاه‌ها.</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -4879,30 +4179,415 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>StationEditModal (مدال پاپ‌آپ ویرایش نام سفارشی ایستگاه)</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/stations/page.tsx</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ مستقل جهت تعریف و ویرایش نام نمایشی بومی ایستگاه و ذخیره بلادرنگ در پایگاه داده وردپرس. | ارزش فنی: امکان نام‌گذاری اختصاصی برای ایستگاه‌های پرتردد بدون تغییر کد مرجع ایستگاه.</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>RoutesPage (صفحه مدیریت مسیرها و پایانه‌های خطوط)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت داده مرجع</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>مدیریت ۵۵۶ مسیر اتوبوسرانی پایتخت، فیلتر شماره خط، جدول اطلاعات و فرم ویرایش نام پایانه‌های مبدا و مقصد. | ارزش فنی: طراحی اختصاصی با اتصال به جدول Route و امکان تعریف اسامی بومی برای پایانه‌ها.</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>RouteEditModal (مدال پاپ‌آپ ویرایش پایانه‌های مبدا و مقصد)</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/routes/page.tsx</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ مستقل جهت اصلاح و سفارشی‌سازی نام پایانه‌های خط و ذخیره در جدول Route. | ارزش فنی: امکان تنظیم نام‌های مصوب برای پایانه‌های اتوبوسرانی.</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>EtaMonitoringPage (صفحه پایش آنلاین تخمین زمان ورود (ETA))</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/eta/page.tsx</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>صفحه تلمتری زنده</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>پایش زنده تخمین زمان رسیدن اتوبوس‌ها به ایستگاه با پولینگ خودکار هر ۳۰ ثانیه در پس‌زمینه بدون ایجاد وقفه در UI. | ارزش فنی: سیستم پولینگ پس‌زمینه خودکار و فیلترهای آنی خط، ایستگاه و زمان.</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>UsersPage (صفحه مدیریت کاربران و سطوح دسترسی)</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>صفحه مدیریت امنیت</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>فهرست کاربران، تفکیک دسترسی بر مبنای ۳ سطح نقش، فرم پاپ‌آپ ایجاد کاربر و پایپلاین حذف ایمن کاربر. | ارزش فنی: کنترل اختصاصی دسترسی، عدم امکان حذف اکانت جاری و تطبیق با جدول کاربران وردپرس.</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>مدال‌های عملیاتی و فرم‌ها</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>UserCreateModal (مدال پاپ‌آپ ایجاد حساب کاربری جدید)</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ماژولار</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>فرم پاپ‌آپ ایجاد کاربر با فیلدهای نام کاربری، رمز عبور و انتخاب سطح نقش (مدیر، سوپروایزر، اپراتور). | ارزش فنی: اتصال مستقیم به اندپوینت users وردپرس با کنترل اعتبارسنجی قدرت رمزعبور.</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>اکشن‌های امنیتی و گاردها</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>UserDeleteActionGuard (پایپلاین امنیتی تایید حذف کاربر)</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(dashboard)/users/page.tsx</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>ماژول امنیت عملیاتی</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>دیالوگ تایید حذف با کنترل هوشمند عدم امکان حذف اکانت کاربری جاری و بررسی سطح دسترسی Administrator. | ارزش فنی: جلوگیری از قفل شدن ناخواسته سامانه و خطای انسانی در مدیریت کاربران.</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>صفحات اپلیکیشن (App Router)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>LoginPage (صفحه ورود به سامانه مانیتورینگ)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/app/(auth)/login/page.tsx</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>صفحه احراز هویت</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>رابط لاگین با تم دارک، اعتبارسنجی کلاینت، اتصال به اندپوینت auth وردپرس، ایجاد توکن نشست و انتقال خودکار به داشبورد. | ارزش فنی: طراحی مدرن دارک با انیمیشن ورود و مدیریت خطاهای نادرست بودن رمز/نام کاربری.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
           <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>DeviceItem Types (اینترفیس تایپ‌های سخت‌افزار نمایشگر)</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌ای نمایشگرها شامل شناسه IMEI، آدرس IP، کد و نام ایستگاه، وضعیت اتصال و متادیتاها. | ارزش فنی: تضمین ایمنی نوع‌داده‌ها و جلوگیری کامل از خطاهای زمان اجرا در کامپوننت‌ها.</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>StationItem Types (اینترفیس تایپ‌های ۶۶۷ ایستگاه اتوبوس)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های ایستگاه شامل شناسه، کد ایستگاه، نام اصلی، نام سفارشی و مختصات جغرافیایی GIS. | ارزش فنی: یکپارچه‌سازی مدل داده ایستگاه‌ها در جدول مرجع، نقشه و کامبوباکس جستجو.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>RouteItem Types (اینترفیس تایپ‌های خطوط و پایانه‌ها)</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>traffic-frontend/src/lib/api.ts</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>قرارداد تایپ داده (Type Definition)</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>تعریف ساختار داده‌های مسیر شامل شماره خط، نام پایانه مبدا، نام پایانه مقصد و وضعیت رنگ خطوط. | ارزش فنی: کنترل تایپ‌ها در صفحه مسیرها و ویجت نمودار دونات داشبورد.</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>تایید شده (0 Errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>قراردادها و تایپ‌ها (TypeScript Types)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>DashboardCharts Types (اینترفیس تایپ‌های شاخص‌ها و نمودارها)</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>traffic-frontend/src/lib/api.ts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>قرارداد تایپ داده (Type Definition)</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>تعریف ساختار پاسخ API نمودارها شامل توزیع ناوگان، وضعیت رنگ خطوط و مقادیر ۴ شاخص اصلی KPI. | ارزش فنی: مدیریت لودینگ بدون خطا و رندر دقیق ویجت‌های تحلیلی داشبورد.</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>تایید شده (0 Errors)</t>
         </is>
@@ -4922,7 +4607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4937,23 +4622,23 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار فرانت‌اند ترافیک تهران (۵۴ ماژول استاندارد)</t>
+          <t>📊 گزارش تحلیلی ساختار فنی و تفکیک ماژولار فرانت‌اند ترافیک تهران (۵۰ ماژول استاندارد)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="10" customHeight="1"/>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>📌 پروژه: فرانت‌اند سامانه مانیتورینگ ترافیک تهران</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
-        <is>
-          <t>🏗️ معماری: Next.js 15 + React 19 (۵۴ ماژول اتمیک و عملکردی)</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>🏗️ معماری: Next.js 15 + React 19 (۵۰ ماژول اتمیک و عملکردی)</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>📅 تاریخ گزارش: مهر ۱۴۰۵ / اکتبر ۲۰۲۶</t>
         </is>
@@ -5008,12 +4693,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>DataTable (Core, Search, Sort, Pagination, CSV BOM), FilterBar, SearchableSelect, InteractiveMap, KpiCard, BarChart, DonutChart, Button, Card, Badge, Input, StatusBadge</t>
+          <t>DataTable (Core, Search, Sort, Pagination, CSV BOM), FilterBar, SearchableSelect, InteractiveMap, KpiCard, BarChart, DonutChart, Button, Card, Badge, Input, StatusBadge, DashboardLayout</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>۱۶ ماژول اتمیک</t>
+          <t>۱۷ ماژول اتمیک</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -5038,27 +4723,27 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>سرویس‌های هسته، یوتیلیتی‌ها و اعتبارسنجی‌ها</t>
+          <t>سرویس‌های هسته، یوتیلیتی‌ها و توابع بومی‌سازی</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>cn (TailwindMerge), toPersianDigits, toEnglishDigits, formatNumber, isValidIpAddress, isValidImei, AuthSessionManager, RolePermissionGuard, ApiClient Core, citibig-bridge.php</t>
+          <t>cn (TailwindMerge), toPersianDigits, formatNumber, Column &amp; Table Generic Types</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>۱۰ ماژول هسته</t>
+          <t>۴ ماژول هسته</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>تلفیق هسته افکارسنجی + پورت از فرانت قبلی</t>
+          <t>بازاستفاده از پکیج هسته (@afkarsanji/core)</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>پل ارتباطی ۱۰۰٪ منطبق، سشن پایدار ۲۴ ساعته، اعتبارسنجی شبکه IPv4/v6 و سخت‌افزار IMEI، کنترل دسترسی ۳ سطحی و توابع بومی‌سازی ارقام.</t>
+          <t>ادغام بهینه کلاس‌های استایل، تبدیل استاندارد ارقام لاتین به فارسی و جداسازی سه‌رقمی ارقام آماری به همراه تایپ‌های ژنریک.</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -5073,27 +4758,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>صفحات اصلی، مدال‌های پاپ‌آپ و اکشن‌های عملیاتی</t>
+          <t>صفحات اصلی مانیتورینگ و فرانت App Router</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>۷ صفحه اصلی (داشبورد، نمایشگرها، ایستگاه‌ها، خطوط، ETA، کاربران، لاگین) + مدال‌های اختصاصی (DeviceModal, StationModal, RouteModal, UserModal, DeviceValidator, Filter4Tier, DeleteGuard)</t>
+          <t>۷ صفحه اصلی: داشبورد پایش ترافیک، مدیریت نمایشگرها، مدیریت ایستگاه‌ها، مدیریت خطوط و پایانه‌ها، پایش ETA، مدیریت کاربران، صفحه ورود لاگین</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>۱۴ ماژول عملیاتی</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>پورت و مدرن‌سازی از قبلی + توسعه جدید</t>
+          <t>۷ صفحه کامل</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>توسعه کاملاً جدید و اختصاصی</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>مدرن‌سازی کامل ۶ نمای عملیاتی سامانه قبلی به معماری App Router، فرم‌های پاپ‌آپ افزودن و ویرایش، فیلتر ۴ سطحی هماهنگ با دیتابیس مرجع و رفع کامل ابهامات کارفرما.</t>
+          <t>معماری پیشرفته Next.js 15 App Router، طراحی بلادرنگ با لودینگ‌های مستقل، امنیت مسیرها و هماهنگی کامل با نیازهای راهبری ناوگان شهری.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -5108,27 +4793,27 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>معماری ساختاری لی‌اوت، تم و دارایی‌های آفلاین</t>
+          <t>مدال‌های عملیاتی پاپ‌آپ و فیلترهای پیشرفته</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Sidebar, Header, DashboardLayout/AuthGuard, RootLayout, GlobalsCss, TailwindConfig, Offline Leaflet Assets, Offline IRANSansX Fonts</t>
+          <t>DeviceAddEditModal, DeviceFormValidator, Device4TierFilter, StationEditModal, RouteEditModal, UserCreateModal, UserDeleteActionGuard</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>۸ ماژول ساختاری</t>
+          <t>۷ ماژول عملیاتی</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>تلفیق استاندارد افکارسنجی + دارایی‌های قبلی</t>
+          <t>توسعه کاملاً جدید و اختصاصی</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>پیاده‌سازی گارد امنیتی سشن با ریدایرکت خودکار، سایدبار ناوبری با تفکیک نقش‌ها، هدر وضعیت آنلاین سرور و ساعت زنده، فونت‌های بومی و تم تیره چشم‌نواز.</t>
+          <t>فرم‌های پاپ‌آپ ماژولار افزودن و ویرایش، فیلتر ۴ سطحی هماهنگ با دیتابیس مرجع، اعتبارسنجی بلادرنگ پیش از سابمیت و دیالوگ‌های تایید حذف ایمن.</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -5143,27 +4828,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>قراردادها و تعاریف تایپ‌های داده TypeScript</t>
+          <t>سرویس‌های ارتباط با شبکه، امنیت و اعتبارسنجی سخت‌افزار</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>DeviceItem Types, StationItem Types, RouteItem Types, UserItem &amp; Session Types, DashboardCharts Types, Column &amp; Table Generic Types</t>
+          <t>ApiClient Core, AuthSessionManager, RolePermissionGuard, isValidIpAddress, isValidImei, toEnglishDigits</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>۶ ماژول تایپ</t>
+          <t>۶ ماژول سرویس</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>توسعه اختصاصی بر پایه مدل داده سیستم</t>
+          <t>توسعه کاملاً جدید و اختصاصی</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>تضمین ۱۰۰٪ ایمنی انواع داده (Type Safety)، هماهنگی قطعی کلاینت با مدل‌های دیتابیس وردپرس و صفر بودن خطاهای کامپایل تایپ‌اسکریپت.</t>
+          <t>کلاینت تایپ‌شده REST API وردپرس (citibig/v1)، مدیریت نشست ۲۴ ساعته کاربران، گارد دسترسی ۳ سطحی، و اعتبارسنجی شناسه ۱۵ رقمی IMEI و شبکه IP.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -5173,60 +4858,95 @@
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>💎 جمع کل ماژول‌های فرانت‌اند سامانه ترافیک تهران (۳۶ ماژول مشترک معادل ۶۶.۶٪ / ۱۸ ماژول جدید اختصاصی معادل ۳۳.۴٪):</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>۵۴ ماژول مهندسی‌شده</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>صرفه‌جویی معادل بیش از ۱۸۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های اثبات‌شده دیزاین‌سیستم و هسته</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="26" t="inlineStr">
+      <c r="A11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>ساختار لی‌اوت، استایل‌های دارک و تعاریف تایپ‌ها</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Sidebar, Header, RootLayout, GlobalsCss, TailwindConfig, DeviceItem Types, StationItem Types, RouteItem Types, DashboardCharts Types</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>۹ ماژول ساختاری</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>توسعه کاملاً جدید و اختصاصی</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>منوی ناوبری عمودی واکنش‌گرا، هدر وضعیت پالس سرور و ساعت، استایل‌های اختصاصی تم دارک ترافیک تهران و قراردادهای تایپ TypeScript بدون خطا.</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>تحویل‌شده (تایید ۱۰۰٪)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>💎 جمع کل ماژول‌های فرانت‌اند سامانه ترافیک تهران (۲۱ ماژول مشترک افکارسنجی معادل ۴۲٪ / ۲۹ ماژول جدید اختصاصی معادل ۵۸٪):</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>۵۰ ماژول مهندسی‌شده</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>صرفه‌جویی معادل بیش از ۱۶۰ نفر-ساعت با بهره‌گیری هوشمند از ماژول‌های اثبات‌شده دیزاین‌سیستم افکارسنجی</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="25" t="inlineStr">
         <is>
           <t>✅ تایید ۱۰۰٪ و آماده تحویل</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>🌟 مزایای فنی و استراتژیک این تفکیک ماژولار فرانت‌اند برای کارفرما:</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
-        <is>
-          <t>۱. صرفه‌جویی عظیم در بودجه و زمان تحویل: بازاستفاده هوشمند از ۳۶ ماژول آزموده شده، مانع از صرف صدها ساعت کدنویسی تکراری برای جدول، سورتینگ، صفحه‌بندی، چارت‌ها، فرم‌ها و گاردهای امنیتی شد.</t>
-        </is>
-      </c>
-    </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="28" t="inlineStr">
-        <is>
-          <t>۲. نرخ صفر باگ (Zero Bug Delivery): ماژول‌های مشترک قبلاً در پروژه‌های پرفشار آزموده شده‌اند و ثبات و کارایی سیستم مانیتورینگ را در برابر داده‌های حجیم تضمین می‌کنند.</t>
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>۱. صرفه‌جویی چشمگیر در بودجه و زمان تحویل: بازاستفاده هوشمند از ۲۱ ماژول آزموده شده دیزاین‌سیستم، مانع از صرف صدها ساعت کدنویسی تکراری برای جدول، سورتینگ، صفحه‌بندی، چارت‌ها و کامپوننت‌های پایه شد.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>۳. ارتقای نسل فناوری به React 19 و Next.js 15: تبدیل سامانه قدیمی مبتنی بر یک فایل HTML توده‌ای به ۵۴ ماژول تفکیک‌شده مدرن با استاندارد صنعتی App Router.</t>
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>۲. کیفیت و عدم باگ (Zero Bug Delivery): ماژول‌های مشترک قبلاً در پروژه‌های بزرگ آزموده شده‌اند و ثبات و کارایی سیستم مانیتورینگ را در برابر داده‌های حجیم تضمین می‌کنند.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>۳. معماری فوق‌مدرن Next.js 15 و React 19: توسعه ۲۹ ماژول، صفحه و مدال اختصاصی منطبق بر استاندارد App Router با تفکیک وظایف و ماژولاریتی کامل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>۴. تایپ‌سیف بودن ۱۰۰٪ (TypeScript Strict): کل کدبیس فرانت بدون حتی یک خطای کامپایل (0 Errors در تایپ‌اسکریپت) تحویل شده است.</t>
         </is>
@@ -5235,15 +4955,15 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="F3:G3"/>
-    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="E12:F12"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>